<commit_message>
Add Mars Ore veins
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="490">
   <si>
     <t>Vein ID</t>
   </si>
@@ -749,10 +749,166 @@
     <t>venus_stone</t>
   </si>
   <si>
-    <t>mars_hematite</t>
-  </si>
-  <si>
-    <t>hematite: 100 [1]</t>
+    <t>deep_chromite</t>
+  </si>
+  <si>
+    <t>redstone: 45</t>
+  </si>
+  <si>
+    <t>thorium: 25</t>
+  </si>
+  <si>
+    <t>uraninite: 20</t>
+  </si>
+  <si>
+    <t>cooperite: 25</t>
+  </si>
+  <si>
+    <t>nickel: 25</t>
+  </si>
+  <si>
+    <t>platinum: 15</t>
+  </si>
+  <si>
+    <t>mars_almandine</t>
+  </si>
+  <si>
+    <t>pyrope: 25</t>
+  </si>
+  <si>
+    <t>mars_apatite</t>
+  </si>
+  <si>
+    <t>mars_coal</t>
+  </si>
+  <si>
+    <t>coal: 50 [1]</t>
+  </si>
+  <si>
+    <t>hematite: 50</t>
+  </si>
+  <si>
+    <t>mars_copper</t>
+  </si>
+  <si>
+    <t>chalcopyrite: 65 [1]</t>
+  </si>
+  <si>
+    <t>mars_galena</t>
+  </si>
+  <si>
+    <t>galena: 30 [1]</t>
+  </si>
+  <si>
+    <t>lead: 25</t>
+  </si>
+  <si>
+    <t>mars_gold</t>
+  </si>
+  <si>
+    <t>mars_lubricant</t>
+  </si>
+  <si>
+    <t>soapstone: 30 [1]</t>
+  </si>
+  <si>
+    <t>mars_neodynium</t>
+  </si>
+  <si>
+    <t>bastnasite: 50 [1]</t>
+  </si>
+  <si>
+    <t>mars_nickel</t>
+  </si>
+  <si>
+    <t>garnierite: 25 [1]</t>
+  </si>
+  <si>
+    <t>nickel: 20</t>
+  </si>
+  <si>
+    <t>mars_pitchblende</t>
+  </si>
+  <si>
+    <t>pitchblende: 35 [1]</t>
+  </si>
+  <si>
+    <t>hematite: 25</t>
+  </si>
+  <si>
+    <t>mars_quartzite</t>
+  </si>
+  <si>
+    <t>mars_salt</t>
+  </si>
+  <si>
+    <t>rock_salt: 20 [1]</t>
+  </si>
+  <si>
+    <t>mars_sapphire</t>
+  </si>
+  <si>
+    <t>green_sapphire: 5 [1]</t>
+  </si>
+  <si>
+    <t>bauxite: 20</t>
+  </si>
+  <si>
+    <t>magnetite: 20</t>
+  </si>
+  <si>
+    <t>gold: 55</t>
+  </si>
+  <si>
+    <t>mars_stibnite</t>
+  </si>
+  <si>
+    <t>mars_sulfur</t>
+  </si>
+  <si>
+    <t>mars_tantalite</t>
+  </si>
+  <si>
+    <t>grossular: 30 [1]</t>
+  </si>
+  <si>
+    <t>mars_tungsten</t>
+  </si>
+  <si>
+    <t>scheelite: 45 [2]</t>
+  </si>
+  <si>
+    <t>tungstate: 35</t>
+  </si>
+  <si>
+    <t>bismuth: 90 [1]</t>
+  </si>
+  <si>
+    <t>sulfur: 10</t>
+  </si>
+  <si>
+    <t>cassiterite: 60 [1]</t>
+  </si>
+  <si>
+    <t>surface_hematite</t>
+  </si>
+  <si>
+    <t>surface_nickel_galena</t>
+  </si>
+  <si>
+    <t>sphalerite: 15 [1]</t>
+  </si>
+  <si>
+    <t>silver: 10</t>
+  </si>
+  <si>
+    <t>cobaltite: 10</t>
+  </si>
+  <si>
+    <t>tetrahedrite: 60 [1]</t>
+  </si>
+  <si>
+    <t>redstone: 5</t>
   </si>
   <si>
     <t>glacio_stone</t>
@@ -848,12 +1004,6 @@
     <t>moon_garnierite</t>
   </si>
   <si>
-    <t>garnierite: 25 [1]</t>
-  </si>
-  <si>
-    <t>nickel: 20</t>
-  </si>
-  <si>
     <t>pentlandite: 25 [1]</t>
   </si>
   <si>
@@ -863,12 +1013,6 @@
     <t>green_sapphire: 5</t>
   </si>
   <si>
-    <t>bauxite: 20</t>
-  </si>
-  <si>
-    <t>magnetite: 20</t>
-  </si>
-  <si>
     <t>moon_graphite</t>
   </si>
   <si>
@@ -920,9 +1064,6 @@
     <t>moon_monazite</t>
   </si>
   <si>
-    <t>bastnasite: 50 [1]</t>
-  </si>
-  <si>
     <t>olivine: 1</t>
   </si>
   <si>
@@ -977,9 +1118,6 @@
     <t>moon_sapphire</t>
   </si>
   <si>
-    <t>pyrope: 25</t>
-  </si>
-  <si>
     <t>olivine: 2</t>
   </si>
   <si>
@@ -998,24 +1136,12 @@
     <t>moon_sheldonite</t>
   </si>
   <si>
-    <t>cooperite: 25</t>
-  </si>
-  <si>
-    <t>platinum: 15</t>
-  </si>
-  <si>
-    <t>nickel: 25</t>
-  </si>
-  <si>
     <t>moon_silver</t>
   </si>
   <si>
     <t>silver: 45 [1]</t>
   </si>
   <si>
-    <t>lead: 25</t>
-  </si>
-  <si>
     <t>moon_sphalerite</t>
   </si>
   <si>
@@ -1184,9 +1310,6 @@
     <t>nether_lubricant</t>
   </si>
   <si>
-    <t>soapstone: 30 [1]</t>
-  </si>
-  <si>
     <t>talc: 20 [1]</t>
   </si>
   <si>
@@ -1211,9 +1334,6 @@
     <t>nether_manganese</t>
   </si>
   <si>
-    <t>grossular: 30 [1]</t>
-  </si>
-  <si>
     <t>spessartine: 20 [1]</t>
   </si>
   <si>
@@ -1316,9 +1436,6 @@
     <t>nether_scheelite</t>
   </si>
   <si>
-    <t>scheelite: 45 [2]</t>
-  </si>
-  <si>
     <t>lithium: 20 [1]</t>
   </si>
   <si>
@@ -1328,9 +1445,6 @@
     <t>nether_silver</t>
   </si>
   <si>
-    <t>galena: 30 [1]</t>
-  </si>
-  <si>
     <t>silver: 35 [1]</t>
   </si>
   <si>
@@ -1353,9 +1467,6 @@
   </si>
   <si>
     <t>pyrite: 35 [1]</t>
-  </si>
-  <si>
-    <t>sphalerite: 15 [1]</t>
   </si>
   <si>
     <t>nether_sylvite</t>
@@ -6113,10 +6224,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AC26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.822014808654785" customWidth="1" style="3"/>
+    <col min="1" max="1" width="20.848892211914062" customWidth="1" style="3"/>
     <col min="2" max="2" width="14.972405433654785" customWidth="1" style="3"/>
     <col min="3" max="3" width="9.140625" customWidth="1" style="3"/>
     <col min="4" max="4" width="9.140625" customWidth="1" style="3"/>
@@ -6125,11 +6236,11 @@
     <col min="7" max="7" width="9.140625" customWidth="1" style="3"/>
     <col min="8" max="8" width="9.140625" customWidth="1" style="3"/>
     <col min="9" max="9" width="9.140625" customWidth="1" style="3"/>
-    <col min="10" max="10" width="16.645116806030273" customWidth="1" style="3"/>
-    <col min="11" max="11" width="9.140625" customWidth="1" style="3"/>
-    <col min="12" max="12" width="9.140625" customWidth="1" style="3"/>
-    <col min="13" max="13" width="9.140625" customWidth="1" style="3"/>
-    <col min="14" max="14" width="9.140625" customWidth="1" style="3"/>
+    <col min="10" max="10" width="20.201292037963867" customWidth="1" style="3"/>
+    <col min="11" max="11" width="23.763607025146484" customWidth="1" style="3"/>
+    <col min="12" max="12" width="19.039091110229492" customWidth="1" style="3"/>
+    <col min="13" max="13" width="18.38944435119629" customWidth="1" style="3"/>
+    <col min="14" max="14" width="12.393258094787598" customWidth="1" style="3"/>
     <col min="15" max="15" width="9.140625" customWidth="1" style="3"/>
     <col min="16" max="16" width="9.140625" customWidth="1" style="3"/>
     <col min="17" max="17" width="9.140625" customWidth="1" style="3"/>
@@ -6248,23 +6359,29 @@
         <v>42</v>
       </c>
       <c r="C2" s="3">
-        <v>210</v>
+        <v>370</v>
       </c>
       <c r="D2" s="3">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E2" s="3">
-        <v>-16</v>
+        <v>-20</v>
       </c>
       <c r="F2" s="3">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>245</v>
       </c>
+      <c r="K2" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="O2" s="1" t="s">
         <v>37</v>
       </c>
@@ -6277,23 +6394,23 @@
       <c r="R2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="1" t="s">
-        <v>37</v>
+      <c r="S2" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="U2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>37</v>
+      <c r="U2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="Y2" s="1" t="s">
         <v>37</v>
@@ -6301,13 +6418,1918 @@
       <c r="Z2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AA2" s="1" t="s">
-        <v>37</v>
+      <c r="AA2" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="AB2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AC2" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="3">
+        <v>370</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="E3" s="3">
+        <v>-20</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
+        <v>60</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="3">
+        <v>370</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="E4" s="3">
+        <v>-20</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>60</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="3">
+        <v>280</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.35</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3">
+        <v>70</v>
+      </c>
+      <c r="G5" s="3">
+        <v>65</v>
+      </c>
+      <c r="H5" s="3">
+        <v>8</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="3">
+        <v>220</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>70</v>
+      </c>
+      <c r="G6" s="3">
+        <v>45</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC6" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="3">
+        <v>215</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>70</v>
+      </c>
+      <c r="G7" s="3">
+        <v>55</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC7" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="3">
+        <v>220</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>70</v>
+      </c>
+      <c r="G8" s="3">
+        <v>50</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="3">
+        <v>215</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>70</v>
+      </c>
+      <c r="G9" s="3">
+        <v>50</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="3">
+        <v>210</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>70</v>
+      </c>
+      <c r="G10" s="3">
+        <v>40</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC10" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="3">
+        <v>220</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3">
+        <v>70</v>
+      </c>
+      <c r="G11" s="3">
+        <v>30</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC11" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="3">
+        <v>215</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>70</v>
+      </c>
+      <c r="G12" s="3">
+        <v>45</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC12" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="3">
+        <v>250</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>70</v>
+      </c>
+      <c r="G13" s="3">
+        <v>55</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC13" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="3">
+        <v>220</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.55</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>70</v>
+      </c>
+      <c r="G14" s="3">
+        <v>20</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC14" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="3">
+        <v>210</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>70</v>
+      </c>
+      <c r="G15" s="3">
+        <v>40</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC15" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="3">
+        <v>210</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>70</v>
+      </c>
+      <c r="G16" s="3">
+        <v>40</v>
+      </c>
+      <c r="H16" s="3">
+        <v>6</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC16" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="3">
+        <v>230</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>70</v>
+      </c>
+      <c r="G17" s="3">
+        <v>40</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC17" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="3">
+        <v>210</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>70</v>
+      </c>
+      <c r="G18" s="3">
+        <v>40</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC18" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="3">
+        <v>215</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>70</v>
+      </c>
+      <c r="G19" s="3">
+        <v>45</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC19" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="3">
+        <v>230</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>70</v>
+      </c>
+      <c r="G20" s="3">
+        <v>42</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC20" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="3">
+        <v>280</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="E21" s="3">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>70</v>
+      </c>
+      <c r="G21" s="3">
+        <v>50</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="V21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC21" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="3">
+        <v>140</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E22" s="3">
+        <v>80</v>
+      </c>
+      <c r="F22" s="3">
+        <v>180</v>
+      </c>
+      <c r="G22" s="3">
+        <v>45</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC22" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="3">
+        <v>135</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E23" s="3">
+        <v>80</v>
+      </c>
+      <c r="F23" s="3">
+        <v>180</v>
+      </c>
+      <c r="G23" s="3">
+        <v>45</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC23" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="3">
+        <v>140</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E24" s="3">
+        <v>80</v>
+      </c>
+      <c r="F24" s="3">
+        <v>180</v>
+      </c>
+      <c r="G24" s="3">
+        <v>45</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC24" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="3">
+        <v>150</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E25" s="3">
+        <v>80</v>
+      </c>
+      <c r="F25" s="3">
+        <v>180</v>
+      </c>
+      <c r="G25" s="3">
+        <v>45</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC25" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="3">
+        <v>140</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E26" s="3">
+        <v>80</v>
+      </c>
+      <c r="F26" s="3">
+        <v>180</v>
+      </c>
+      <c r="G26" s="3">
+        <v>45</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC26" s="1" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6415,16 +8437,16 @@
         <v>19</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>246</v>
+        <v>298</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>247</v>
+        <v>299</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>248</v>
+        <v>300</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>26</v>
@@ -6432,7 +8454,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>249</v>
+        <v>301</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>42</v>
@@ -6453,16 +8475,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>250</v>
+        <v>302</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>90</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>251</v>
+        <v>303</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>36</v>
@@ -6497,7 +8519,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>253</v>
+        <v>305</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>42</v>
@@ -6518,13 +8540,13 @@
         <v>50</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>254</v>
+        <v>306</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>255</v>
+        <v>307</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>256</v>
+        <v>308</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>36</v>
@@ -6559,7 +8581,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>98</v>
@@ -6583,16 +8605,16 @@
         <v>10</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>259</v>
+        <v>311</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>260</v>
+        <v>312</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>211</v>
@@ -6630,7 +8652,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>261</v>
+        <v>313</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>42</v>
@@ -6651,16 +8673,16 @@
         <v>40</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>262</v>
+        <v>314</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>263</v>
+        <v>315</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>264</v>
+        <v>316</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>265</v>
+        <v>317</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>36</v>
@@ -6695,7 +8717,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>266</v>
+        <v>318</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>42</v>
@@ -6716,16 +8738,16 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>267</v>
+        <v>319</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>268</v>
+        <v>320</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>269</v>
+        <v>321</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>270</v>
+        <v>322</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>37</v>
@@ -6760,7 +8782,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -6784,16 +8806,16 @@
         <v>7</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>273</v>
+        <v>325</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>274</v>
+        <v>326</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>275</v>
+        <v>327</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>37</v>
@@ -6828,7 +8850,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>276</v>
+        <v>328</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>42</v>
@@ -6849,16 +8871,16 @@
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>124</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>279</v>
+        <v>329</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>126</v>
@@ -6896,7 +8918,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>280</v>
+        <v>330</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -6920,13 +8942,13 @@
         <v>10</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>130</v>
@@ -6964,7 +8986,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>284</v>
+        <v>332</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>98</v>
@@ -6988,13 +9010,13 @@
         <v>12</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>285</v>
+        <v>333</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>286</v>
+        <v>334</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>287</v>
+        <v>335</v>
       </c>
       <c r="O10" s="2" t="s">
         <v>36</v>
@@ -7029,7 +9051,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>288</v>
+        <v>336</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -7056,16 +9078,16 @@
         <v>136</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>289</v>
+        <v>337</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>201</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>290</v>
+        <v>338</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>36</v>
@@ -7100,7 +9122,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>291</v>
+        <v>339</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>42</v>
@@ -7168,7 +9190,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>292</v>
+        <v>340</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>42</v>
@@ -7189,13 +9211,13 @@
         <v>70</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>293</v>
+        <v>341</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>59</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>294</v>
+        <v>342</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>61</v>
@@ -7236,7 +9258,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>295</v>
+        <v>343</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>42</v>
@@ -7301,7 +9323,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>296</v>
+        <v>344</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>42</v>
@@ -7322,7 +9344,7 @@
         <v>35</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>297</v>
+        <v>345</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>170</v>
@@ -7331,10 +9353,10 @@
         <v>171</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>298</v>
+        <v>346</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>36</v>
@@ -7369,7 +9391,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>299</v>
+        <v>347</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>42</v>
@@ -7399,7 +9421,7 @@
         <v>66</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>36</v>
@@ -7434,7 +9456,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>300</v>
+        <v>348</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>42</v>
@@ -7455,7 +9477,7 @@
         <v>50</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>301</v>
+        <v>266</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>175</v>
@@ -7464,7 +9486,7 @@
         <v>176</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>302</v>
+        <v>349</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>37</v>
@@ -7499,7 +9521,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>303</v>
+        <v>350</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>42</v>
@@ -7520,16 +9542,16 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>304</v>
+        <v>351</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>305</v>
+        <v>352</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>306</v>
+        <v>353</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>307</v>
+        <v>354</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>37</v>
@@ -7564,7 +9586,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>308</v>
+        <v>355</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>42</v>
@@ -7585,16 +9607,16 @@
         <v>60</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>309</v>
+        <v>356</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>310</v>
+        <v>357</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>311</v>
+        <v>358</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>37</v>
@@ -7629,7 +9651,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>313</v>
+        <v>360</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>42</v>
@@ -7659,7 +9681,7 @@
         <v>191</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>37</v>
@@ -7694,7 +9716,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>314</v>
+        <v>361</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>42</v>
@@ -7715,16 +9737,16 @@
         <v>35</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>315</v>
+        <v>362</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>316</v>
+        <v>363</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>317</v>
+        <v>364</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>318</v>
+        <v>365</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>37</v>
@@ -7759,7 +9781,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>319</v>
+        <v>366</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -7786,7 +9808,7 @@
         <v>71</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>320</v>
+        <v>252</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>73</v>
@@ -7795,7 +9817,7 @@
         <v>74</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>321</v>
+        <v>367</v>
       </c>
       <c r="O22" s="2" t="s">
         <v>36</v>
@@ -7830,7 +9852,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>322</v>
+        <v>368</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>42</v>
@@ -7851,13 +9873,13 @@
         <v>20</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>323</v>
+        <v>369</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>324</v>
+        <v>370</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>325</v>
+        <v>371</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>36</v>
@@ -7892,7 +9914,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>326</v>
+        <v>372</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>42</v>
@@ -7916,13 +9938,13 @@
         <v>80</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>327</v>
+        <v>248</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>328</v>
+        <v>250</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>329</v>
+        <v>249</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>37</v>
@@ -7957,7 +9979,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>42</v>
@@ -7981,13 +10003,13 @@
         <v>203</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>331</v>
+        <v>374</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>332</v>
+        <v>261</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>36</v>
@@ -8022,7 +10044,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>333</v>
+        <v>375</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>42</v>
@@ -8043,10 +10065,10 @@
         <v>40</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>334</v>
+        <v>376</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>335</v>
+        <v>377</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>216</v>
@@ -8084,7 +10106,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>336</v>
+        <v>378</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>42</v>
@@ -8105,16 +10127,16 @@
         <v>40</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>337</v>
+        <v>379</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>338</v>
+        <v>380</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>221</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>339</v>
+        <v>381</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>37</v>
@@ -8149,7 +10171,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>340</v>
+        <v>382</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -8307,16 +10329,16 @@
         <v>11</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>341</v>
+        <v>383</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>342</v>
+        <v>384</v>
       </c>
       <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>343</v>
+        <v>385</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>19</v>
@@ -8333,7 +10355,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>344</v>
+        <v>386</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -8357,7 +10379,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>345</v>
+        <v>387</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>36</v>
@@ -8389,7 +10411,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>346</v>
+        <v>388</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>42</v>
@@ -8410,10 +10432,10 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>348</v>
+        <v>390</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>91</v>
@@ -8448,7 +10470,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>349</v>
+        <v>391</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>31</v>
@@ -8472,13 +10494,13 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>351</v>
+        <v>393</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>352</v>
+        <v>394</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>96</v>
@@ -8513,7 +10535,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>353</v>
+        <v>395</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>98</v>
@@ -8537,13 +10559,13 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>259</v>
+        <v>311</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>260</v>
+        <v>312</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>211</v>
@@ -8578,7 +10600,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>354</v>
+        <v>396</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>42</v>
@@ -8599,10 +10621,10 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>355</v>
+        <v>397</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>356</v>
+        <v>398</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>36</v>
@@ -8634,7 +10656,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>357</v>
+        <v>399</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>42</v>
@@ -8655,16 +10677,16 @@
         <v>45</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>358</v>
+        <v>400</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>113</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>359</v>
+        <v>401</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>360</v>
+        <v>402</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>37</v>
@@ -8696,7 +10718,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>361</v>
+        <v>403</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -8720,16 +10742,16 @@
         <v>8</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>362</v>
+        <v>404</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>33</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>363</v>
+        <v>405</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>364</v>
+        <v>406</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>37</v>
@@ -8761,7 +10783,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>365</v>
+        <v>407</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>42</v>
@@ -8782,13 +10804,13 @@
         <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>366</v>
+        <v>408</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>367</v>
+        <v>409</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>368</v>
+        <v>410</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>120</v>
@@ -8823,7 +10845,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>369</v>
+        <v>411</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>42</v>
@@ -8844,16 +10866,16 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>370</v>
+        <v>412</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>279</v>
+        <v>329</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>126</v>
@@ -8888,7 +10910,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>371</v>
+        <v>413</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>42</v>
@@ -8909,10 +10931,10 @@
         <v>37</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>372</v>
+        <v>414</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>373</v>
+        <v>415</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>45</v>
@@ -8950,7 +10972,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>374</v>
+        <v>416</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>42</v>
@@ -9012,7 +11034,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>375</v>
+        <v>417</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>98</v>
@@ -9036,13 +11058,13 @@
         <v>12</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>376</v>
+        <v>418</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>377</v>
+        <v>419</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>378</v>
+        <v>420</v>
       </c>
       <c r="O13" s="2" t="s">
         <v>36</v>
@@ -9074,7 +11096,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>379</v>
+        <v>421</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -9098,16 +11120,16 @@
         <v>9</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>380</v>
+        <v>422</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>381</v>
+        <v>423</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>138</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>290</v>
+        <v>338</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>36</v>
@@ -9139,7 +11161,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>382</v>
+        <v>424</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>42</v>
@@ -9166,7 +11188,7 @@
         <v>49</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>383</v>
+        <v>425</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>51</v>
@@ -9204,7 +11226,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>384</v>
+        <v>426</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>42</v>
@@ -9225,13 +11247,13 @@
         <v>40</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>385</v>
+        <v>427</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>386</v>
+        <v>428</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>387</v>
+        <v>429</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>148</v>
@@ -9266,7 +11288,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>388</v>
+        <v>430</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>42</v>
@@ -9287,16 +11309,16 @@
         <v>41</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>389</v>
+        <v>264</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>390</v>
+        <v>431</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>391</v>
+        <v>432</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>392</v>
+        <v>433</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>157</v>
@@ -9331,7 +11353,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>393</v>
+        <v>434</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>42</v>
@@ -9352,16 +11374,16 @@
         <v>39</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>394</v>
+        <v>435</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>395</v>
+        <v>436</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>162</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>396</v>
+        <v>437</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>62</v>
@@ -9396,7 +11418,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>397</v>
+        <v>438</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>42</v>
@@ -9417,13 +11439,13 @@
         <v>45</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>398</v>
+        <v>284</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>399</v>
+        <v>439</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>400</v>
+        <v>440</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>167</v>
@@ -9458,7 +11480,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>401</v>
+        <v>441</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>42</v>
@@ -9479,13 +11501,13 @@
         <v>41</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>297</v>
+        <v>345</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>402</v>
+        <v>442</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>403</v>
+        <v>443</v>
       </c>
       <c r="O20" s="2" t="s">
         <v>36</v>
@@ -9517,7 +11539,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>404</v>
+        <v>444</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>42</v>
@@ -9544,10 +11566,10 @@
         <v>65</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>405</v>
+        <v>445</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>406</v>
+        <v>446</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>36</v>
@@ -9579,7 +11601,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>407</v>
+        <v>447</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>42</v>
@@ -9600,13 +11622,13 @@
         <v>45</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>408</v>
+        <v>448</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>409</v>
+        <v>449</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="O22" s="2" t="s">
         <v>36</v>
@@ -9638,7 +11660,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>411</v>
+        <v>451</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>42</v>
@@ -9659,10 +11681,10 @@
         <v>32</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>412</v>
+        <v>452</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>413</v>
+        <v>453</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>37</v>
@@ -9694,7 +11716,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>414</v>
+        <v>454</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>42</v>
@@ -9715,13 +11737,13 @@
         <v>31</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>415</v>
+        <v>455</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>416</v>
+        <v>456</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>417</v>
+        <v>457</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>183</v>
@@ -9756,7 +11778,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>418</v>
+        <v>458</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>42</v>
@@ -9812,7 +11834,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>419</v>
+        <v>459</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>42</v>
@@ -9833,13 +11855,13 @@
         <v>45</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>420</v>
+        <v>460</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>421</v>
+        <v>461</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>422</v>
+        <v>462</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>37</v>
@@ -9871,7 +11893,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>423</v>
+        <v>463</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>42</v>
@@ -9895,10 +11917,10 @@
         <v>189</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>424</v>
+        <v>464</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>425</v>
+        <v>465</v>
       </c>
       <c r="O27" s="2" t="s">
         <v>36</v>
@@ -9930,7 +11952,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>426</v>
+        <v>466</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>42</v>
@@ -9951,13 +11973,13 @@
         <v>50</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>315</v>
+        <v>362</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>427</v>
+        <v>467</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>428</v>
+        <v>468</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>201</v>
@@ -9992,7 +12014,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>429</v>
+        <v>469</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -10022,10 +12044,10 @@
         <v>72</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>430</v>
+        <v>470</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>431</v>
+        <v>471</v>
       </c>
       <c r="O29" s="2" t="s">
         <v>36</v>
@@ -10057,7 +12079,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>432</v>
+        <v>472</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>42</v>
@@ -10078,13 +12100,13 @@
         <v>25</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>433</v>
+        <v>286</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>434</v>
+        <v>473</v>
       </c>
       <c r="O30" s="2" t="s">
         <v>36</v>
@@ -10116,7 +12138,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>435</v>
+        <v>474</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>42</v>
@@ -10146,7 +12168,7 @@
         <v>82</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>37</v>
@@ -10178,7 +12200,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>436</v>
+        <v>475</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>42</v>
@@ -10199,13 +12221,13 @@
         <v>45</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>437</v>
+        <v>260</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>438</v>
+        <v>476</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>439</v>
+        <v>477</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>36</v>
@@ -10237,7 +12259,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>440</v>
+        <v>478</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>42</v>
@@ -10258,13 +12280,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>208</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>442</v>
+        <v>480</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>37</v>
@@ -10296,7 +12318,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>443</v>
+        <v>481</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>42</v>
@@ -10317,13 +12339,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>445</v>
+        <v>483</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>446</v>
+        <v>293</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>37</v>
@@ -10355,7 +12377,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>447</v>
+        <v>484</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>42</v>
@@ -10376,7 +12398,7 @@
         <v>17</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>448</v>
+        <v>485</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>36</v>
@@ -10408,7 +12430,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>449</v>
+        <v>486</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>42</v>
@@ -10429,10 +12451,10 @@
         <v>45</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>450</v>
+        <v>487</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>451</v>
+        <v>488</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>221</v>
@@ -10467,7 +12489,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>452</v>
+        <v>489</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
fixed ore veins jsons
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="503">
   <si>
     <t>Vein ID</t>
   </si>
@@ -896,6 +896,9 @@
     <t>tungstate: 35</t>
   </si>
   <si>
+    <t>mars_surface_bismuthinite</t>
+  </si>
+  <si>
     <t>bismuth: 20 [1]</t>
   </si>
   <si>
@@ -908,6 +911,9 @@
     <t>gypsum: 10</t>
   </si>
   <si>
+    <t>mars_surface_cassiterite</t>
+  </si>
+  <si>
     <t>cassiterite: 55 [1]</t>
   </si>
   <si>
@@ -917,19 +923,22 @@
     <t>saltpeter: 10</t>
   </si>
   <si>
-    <t>surface_hematite</t>
+    <t>mars_surface_hematite</t>
   </si>
   <si>
     <t>calcite: 5</t>
   </si>
   <si>
-    <t>surface_nickel_galena</t>
+    <t>mars_surface_nickel_galena</t>
   </si>
   <si>
     <t>silver: 10</t>
   </si>
   <si>
     <t>cobaltite: 10</t>
+  </si>
+  <si>
+    <t>mars_surface_tetrahedrite</t>
   </si>
   <si>
     <t>tetrahedrite: 60 [1]</t>
@@ -6263,7 +6272,7 @@
   <dimension ref="A1:AE27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.774301528930664" customWidth="1" style="3"/>
+    <col min="1" max="1" width="26.277278900146484" customWidth="1" style="3"/>
     <col min="2" max="2" width="14.972405433654785" customWidth="1" style="3"/>
     <col min="3" max="3" width="9.140625" customWidth="1" style="3"/>
     <col min="4" max="4" width="9.140625" customWidth="1" style="3"/>
@@ -8198,7 +8207,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>223</v>
+        <v>293</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -8219,16 +8228,16 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>35</v>
@@ -8284,7 +8293,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>228</v>
+        <v>298</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -8305,13 +8314,13 @@
         <v>45</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="O24" s="2" t="s">
         <v>35</v>
@@ -8367,7 +8376,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -8397,7 +8406,7 @@
         <v>55</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>35</v>
@@ -8453,7 +8462,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -8483,10 +8492,10 @@
         <v>204</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="O26" s="2" t="s">
         <v>35</v>
@@ -8542,7 +8551,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>240</v>
+        <v>307</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -8563,7 +8572,7 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>242</v>
@@ -8572,7 +8581,7 @@
         <v>222</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="O27" s="2" t="s">
         <v>35</v>
@@ -8730,16 +8739,16 @@
         <v>19</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>26</v>
@@ -8747,7 +8756,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -8768,16 +8777,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>35</v>
@@ -8812,7 +8821,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -8833,13 +8842,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>35</v>
@@ -8874,7 +8883,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>99</v>
@@ -8898,16 +8907,16 @@
         <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>212</v>
@@ -8945,7 +8954,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>31</v>
@@ -8966,16 +8975,16 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>35</v>
@@ -9010,7 +9019,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -9075,7 +9084,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -9096,16 +9105,16 @@
         <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>36</v>
@@ -9140,7 +9149,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>38</v>
@@ -9164,16 +9173,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>36</v>
@@ -9208,7 +9217,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -9238,7 +9247,7 @@
         <v>125</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>127</v>
@@ -9276,7 +9285,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>38</v>
@@ -9306,7 +9315,7 @@
         <v>268</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>131</v>
@@ -9344,7 +9353,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>99</v>
@@ -9368,13 +9377,13 @@
         <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>35</v>
@@ -9409,7 +9418,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -9436,16 +9445,16 @@
         <v>137</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>202</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="O12" s="2" t="s">
         <v>35</v>
@@ -9480,7 +9489,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -9548,7 +9557,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -9569,13 +9578,13 @@
         <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>63</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>65</v>
@@ -9616,7 +9625,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -9681,7 +9690,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -9702,7 +9711,7 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>171</v>
@@ -9711,10 +9720,10 @@
         <v>172</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>35</v>
@@ -9749,7 +9758,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -9779,7 +9788,7 @@
         <v>70</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="O17" s="2" t="s">
         <v>35</v>
@@ -9814,7 +9823,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -9844,7 +9853,7 @@
         <v>177</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>36</v>
@@ -9879,7 +9888,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -9900,16 +9909,16 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>36</v>
@@ -9944,7 +9953,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -9965,16 +9974,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>36</v>
@@ -10009,7 +10018,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -10039,7 +10048,7 @@
         <v>192</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>36</v>
@@ -10074,7 +10083,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -10095,16 +10104,16 @@
         <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>36</v>
@@ -10139,7 +10148,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
@@ -10175,7 +10184,7 @@
         <v>79</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>35</v>
@@ -10210,7 +10219,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -10231,13 +10240,13 @@
         <v>20</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="O24" s="2" t="s">
         <v>35</v>
@@ -10272,7 +10281,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -10296,13 +10305,13 @@
         <v>204</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>265</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>35</v>
@@ -10337,7 +10346,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -10358,13 +10367,13 @@
         <v>35</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>36</v>
@@ -10399,7 +10408,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -10420,16 +10429,16 @@
         <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>222</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>36</v>
@@ -10464,7 +10473,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
@@ -10622,16 +10631,16 @@
         <v>11</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>19</v>
@@ -10648,7 +10657,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -10672,7 +10681,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>35</v>
@@ -10704,7 +10713,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -10725,10 +10734,10 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>92</v>
@@ -10763,7 +10772,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -10787,13 +10796,13 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>97</v>
@@ -10828,7 +10837,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>99</v>
@@ -10852,13 +10861,13 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>212</v>
@@ -10893,7 +10902,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -10914,10 +10923,10 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>35</v>
@@ -10949,7 +10958,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -11011,7 +11020,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -11032,16 +11041,16 @@
         <v>45</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>114</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>36</v>
@@ -11073,7 +11082,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>38</v>
@@ -11097,16 +11106,16 @@
         <v>8</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>36</v>
@@ -11138,7 +11147,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -11159,13 +11168,13 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>121</v>
@@ -11200,7 +11209,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -11227,10 +11236,10 @@
         <v>277</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>127</v>
@@ -11265,7 +11274,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>31</v>
@@ -11286,10 +11295,10 @@
         <v>37</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>49</v>
@@ -11327,7 +11336,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -11389,7 +11398,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>99</v>
@@ -11413,13 +11422,13 @@
         <v>12</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>35</v>
@@ -11451,7 +11460,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
@@ -11475,16 +11484,16 @@
         <v>9</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>139</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>35</v>
@@ -11516,7 +11525,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -11543,7 +11552,7 @@
         <v>53</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>55</v>
@@ -11581,7 +11590,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -11602,13 +11611,13 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>149</v>
@@ -11643,7 +11652,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -11667,13 +11676,13 @@
         <v>272</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>158</v>
@@ -11708,7 +11717,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -11729,16 +11738,16 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>163</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>66</v>
@@ -11773,7 +11782,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -11797,10 +11806,10 @@
         <v>290</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>168</v>
@@ -11835,7 +11844,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -11856,13 +11865,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>35</v>
@@ -11894,7 +11903,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -11921,10 +11930,10 @@
         <v>69</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="O22" s="2" t="s">
         <v>35</v>
@@ -11956,7 +11965,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -11977,13 +11986,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>35</v>
@@ -12015,7 +12024,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -12036,7 +12045,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>36</v>
@@ -12068,7 +12077,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -12089,13 +12098,13 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>184</v>
@@ -12130,7 +12139,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -12189,7 +12198,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -12210,13 +12219,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>36</v>
@@ -12248,7 +12257,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -12272,10 +12281,10 @@
         <v>190</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="O28" s="2" t="s">
         <v>35</v>
@@ -12307,7 +12316,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -12328,13 +12337,13 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>202</v>
@@ -12369,7 +12378,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
@@ -12399,10 +12408,10 @@
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="O30" s="2" t="s">
         <v>35</v>
@@ -12434,7 +12443,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -12455,13 +12464,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>82</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>35</v>
@@ -12493,7 +12502,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -12517,10 +12526,10 @@
         <v>264</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>35</v>
@@ -12552,7 +12561,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -12573,13 +12582,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>209</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>36</v>
@@ -12611,7 +12620,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -12632,13 +12641,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>36</v>
@@ -12670,7 +12679,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -12691,7 +12700,7 @@
         <v>17</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>35</v>
@@ -12723,7 +12732,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -12744,10 +12753,10 @@
         <v>45</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>222</v>
@@ -12782,7 +12791,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
add more trona to mars lube vein
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="514">
   <si>
     <t>Vein ID</t>
   </si>
@@ -851,532 +851,535 @@
     <t>mars_lubricant</t>
   </si>
   <si>
-    <t>soapstone: 10</t>
+    <t>soapstone: 15</t>
+  </si>
+  <si>
+    <t>talc: 15</t>
+  </si>
+  <si>
+    <t>glauconite_sand: 5</t>
+  </si>
+  <si>
+    <t>trona: 25</t>
+  </si>
+  <si>
+    <t>pentlandite: 5</t>
+  </si>
+  <si>
+    <t>mars_neodynium</t>
+  </si>
+  <si>
+    <t>bastnasite: 50 [1]</t>
+  </si>
+  <si>
+    <t>mars_nickel</t>
+  </si>
+  <si>
+    <t>garnierite: 25 [1]</t>
+  </si>
+  <si>
+    <t>nickel: 20</t>
+  </si>
+  <si>
+    <t>mars_pitchblende</t>
+  </si>
+  <si>
+    <t>pitchblende: 35 [1]</t>
+  </si>
+  <si>
+    <t>hematite: 25</t>
+  </si>
+  <si>
+    <t>mars_quartzite</t>
+  </si>
+  <si>
+    <t>mars_salt</t>
+  </si>
+  <si>
+    <t>rock_salt: 20 [1]</t>
+  </si>
+  <si>
+    <t>mars_stibnite</t>
+  </si>
+  <si>
+    <t>mars_sulfur</t>
+  </si>
+  <si>
+    <t>sulfur: 15</t>
+  </si>
+  <si>
+    <t>pyrite: 45</t>
+  </si>
+  <si>
+    <t>sphalerite: 25</t>
+  </si>
+  <si>
+    <t>mars_tantalite</t>
+  </si>
+  <si>
+    <t>grossular: 10</t>
+  </si>
+  <si>
+    <t>spessartine: 10</t>
+  </si>
+  <si>
+    <t>pyrolusite: 40 [1]</t>
+  </si>
+  <si>
+    <t>tantalite: 35 [1]</t>
+  </si>
+  <si>
+    <t>mars_tungsten</t>
+  </si>
+  <si>
+    <t>tungstate: 35</t>
+  </si>
+  <si>
+    <t>mars_surface_bismuthinite</t>
+  </si>
+  <si>
+    <t>bismuth: 20 [1]</t>
+  </si>
+  <si>
+    <t>sulfur: 10</t>
+  </si>
+  <si>
+    <t>gypsum: 10</t>
+  </si>
+  <si>
+    <t>mars_surface_cassiterite</t>
+  </si>
+  <si>
+    <t>cassiterite: 55 [1]</t>
+  </si>
+  <si>
+    <t>tin: 35</t>
+  </si>
+  <si>
+    <t>saltpeter: 10</t>
+  </si>
+  <si>
+    <t>mars_surface_hematite</t>
+  </si>
+  <si>
+    <t>calcite: 5</t>
+  </si>
+  <si>
+    <t>mars_surface_nickel_galena</t>
+  </si>
+  <si>
+    <t>cobaltite: 10</t>
+  </si>
+  <si>
+    <t>mars_surface_tetrahedrite</t>
+  </si>
+  <si>
+    <t>tetrahedrite: 60 [1]</t>
+  </si>
+  <si>
+    <t>redstone: 5</t>
+  </si>
+  <si>
+    <t>glacio_stone</t>
+  </si>
+  <si>
+    <t>moon_deepslate</t>
+  </si>
+  <si>
+    <t>moon_stone</t>
+  </si>
+  <si>
+    <t>moon_apatite</t>
+  </si>
+  <si>
+    <t>apatite: 25</t>
+  </si>
+  <si>
+    <t>pyrochlore: 40 [1]</t>
+  </si>
+  <si>
+    <t>olivine: 5</t>
+  </si>
+  <si>
+    <t>moon_bauxite</t>
+  </si>
+  <si>
+    <t>bauxite: 35 [1]</t>
+  </si>
+  <si>
+    <t>ilmenite: 40 [1]</t>
+  </si>
+  <si>
+    <t>armalcolite: 20</t>
+  </si>
+  <si>
+    <t>moon_beryllium</t>
+  </si>
+  <si>
+    <t>beryllium: 35 [1]</t>
+  </si>
+  <si>
+    <t>emerald: 50 [2]</t>
+  </si>
+  <si>
+    <t>thorium: 1</t>
+  </si>
+  <si>
+    <t>moon_cassiterite</t>
+  </si>
+  <si>
+    <t>chalcopyrite: 30 [1]</t>
+  </si>
+  <si>
+    <t>zeolite: 5</t>
+  </si>
+  <si>
+    <t>cassiterite: 35 [1]</t>
+  </si>
+  <si>
+    <t>tin: 15</t>
+  </si>
+  <si>
+    <t>moon_sheldonite</t>
+  </si>
+  <si>
+    <t>moon_desh</t>
+  </si>
+  <si>
+    <t>desh: 25</t>
+  </si>
+  <si>
+    <t>ilmenite: 30 [1]</t>
+  </si>
+  <si>
+    <t>aluminium: 25</t>
+  </si>
+  <si>
+    <t>moon_garnet</t>
+  </si>
+  <si>
+    <t>red_garnet: 10</t>
+  </si>
+  <si>
+    <t>yellow_garnet: 15</t>
+  </si>
+  <si>
+    <t>amethyst: 40 [1]</t>
+  </si>
+  <si>
+    <t>opal: 40 [1]</t>
+  </si>
+  <si>
+    <t>moon_garnierite</t>
+  </si>
+  <si>
+    <t>pentlandite: 25 [1]</t>
+  </si>
+  <si>
+    <t>moon_gold</t>
+  </si>
+  <si>
+    <t>magnetite: 20</t>
+  </si>
+  <si>
+    <t>moon_graphite</t>
+  </si>
+  <si>
+    <t>graphite: 50 [1]</t>
+  </si>
+  <si>
+    <t>diamond: 35</t>
+  </si>
+  <si>
+    <t>olivine: 10</t>
+  </si>
+  <si>
+    <t>moon_gypsum</t>
+  </si>
+  <si>
+    <t>calcite: 25</t>
+  </si>
+  <si>
+    <t>gypsum: 35 [1]</t>
+  </si>
+  <si>
+    <t>moon_lubricant</t>
+  </si>
+  <si>
+    <t>moon_magnetite</t>
+  </si>
+  <si>
+    <t>magnetite: 25</t>
+  </si>
+  <si>
+    <t>chromite: 40 [2]</t>
+  </si>
+  <si>
+    <t>moon_manganese</t>
+  </si>
+  <si>
+    <t>moon_mica</t>
+  </si>
+  <si>
+    <t>kyanite: 35 [1]</t>
+  </si>
+  <si>
+    <t>aluminium: 15</t>
+  </si>
+  <si>
+    <t>moon_molybdenum</t>
+  </si>
+  <si>
+    <t>moon_monazite</t>
+  </si>
+  <si>
+    <t>olivine: 1</t>
+  </si>
+  <si>
+    <t>moon_pyrolusite</t>
+  </si>
+  <si>
+    <t>pyrolusite: 40 [2]</t>
+  </si>
+  <si>
+    <t>cobaltite: 25</t>
+  </si>
+  <si>
+    <t>cobalt: 25</t>
+  </si>
+  <si>
+    <t>tantalite: 15</t>
+  </si>
+  <si>
+    <t>moon_quartz</t>
+  </si>
+  <si>
+    <t>quartzite: 20</t>
+  </si>
+  <si>
+    <t>certus_quartz: 45 [2]</t>
+  </si>
+  <si>
+    <t>nether_quartz: 30 [1]</t>
+  </si>
+  <si>
+    <t>barite: 5</t>
+  </si>
+  <si>
+    <t>moon_redstone</t>
+  </si>
+  <si>
+    <t>moon_saltpeter</t>
+  </si>
+  <si>
+    <t>saltpeter: 35 [1]</t>
+  </si>
+  <si>
+    <t>soapstone: 25</t>
+  </si>
+  <si>
+    <t>electrotine: 45</t>
+  </si>
+  <si>
+    <t>moon_sapphire</t>
+  </si>
+  <si>
+    <t>olivine: 2</t>
+  </si>
+  <si>
+    <t>moon_scheelite</t>
+  </si>
+  <si>
+    <t>scheelite: 40 [1]</t>
+  </si>
+  <si>
+    <t>tungstate: 50 [2]</t>
+  </si>
+  <si>
+    <t>lithium: 10</t>
+  </si>
+  <si>
+    <t>moon_silver</t>
+  </si>
+  <si>
+    <t>silver: 45 [1]</t>
+  </si>
+  <si>
+    <t>moon_sphalerite</t>
+  </si>
+  <si>
+    <t>desh: 10</t>
+  </si>
+  <si>
+    <t>sphalerite: 50 [1]</t>
+  </si>
+  <si>
+    <t>pyrite: 40</t>
+  </si>
+  <si>
+    <t>moon_tetrahedrite</t>
+  </si>
+  <si>
+    <t>tetrahedrite: 40 [1]</t>
+  </si>
+  <si>
+    <t>copper: 15</t>
+  </si>
+  <si>
+    <t>chalcocite: 25</t>
+  </si>
+  <si>
+    <t>moon_topaz</t>
+  </si>
+  <si>
+    <t>blackstone</t>
+  </si>
+  <si>
+    <t>deepslate</t>
+  </si>
+  <si>
+    <t>dripstone</t>
+  </si>
+  <si>
+    <t>nether_anthracite</t>
+  </si>
+  <si>
+    <t>anthracite: 100</t>
+  </si>
+  <si>
+    <t>nether_apatite</t>
+  </si>
+  <si>
+    <t>apatite: 50 [2]</t>
+  </si>
+  <si>
+    <t>tricalcium_phosphate: 35 [1]</t>
+  </si>
+  <si>
+    <t>nether_basaltic_sands</t>
+  </si>
+  <si>
+    <t>basaltic_mineral_sand: 35 [1]</t>
+  </si>
+  <si>
+    <t>granitic_mineral_sand: 25 [1]</t>
+  </si>
+  <si>
+    <t>fullers_earth: 25 [1]</t>
+  </si>
+  <si>
+    <t>nether_beryllium</t>
+  </si>
+  <si>
+    <t>nether_cassiterite</t>
+  </si>
+  <si>
+    <t>cassiterite: 40 [2]</t>
+  </si>
+  <si>
+    <t>tin: 60 [2]</t>
+  </si>
+  <si>
+    <t>nether_sheldonite</t>
+  </si>
+  <si>
+    <t>nether_copper</t>
+  </si>
+  <si>
+    <t>chalcopyrite: 20 [1]</t>
+  </si>
+  <si>
+    <t>pyrite: 10 [1]</t>
+  </si>
+  <si>
+    <t>copper: 65 [2]</t>
+  </si>
+  <si>
+    <t>nether_garnet</t>
+  </si>
+  <si>
+    <t>red_garnet: 10 [1]</t>
+  </si>
+  <si>
+    <t>amethyst: 40 [2]</t>
+  </si>
+  <si>
+    <t>opal: 40 [2]</t>
+  </si>
+  <si>
+    <t>nether_garnet_tin</t>
+  </si>
+  <si>
+    <t>cassiterite_sand: 35 [1]</t>
+  </si>
+  <si>
+    <t>garnet_sand: 25 [1]</t>
+  </si>
+  <si>
+    <t>asbestos: 25 [1]</t>
+  </si>
+  <si>
+    <t>nether_garnierite</t>
+  </si>
+  <si>
+    <t>cobaltite: 20 [1]</t>
+  </si>
+  <si>
+    <t>nether_goethite</t>
+  </si>
+  <si>
+    <t>goethite: 50 [3]</t>
+  </si>
+  <si>
+    <t>yellow_limonite: 15 [1]</t>
+  </si>
+  <si>
+    <t>nether_gold</t>
+  </si>
+  <si>
+    <t>nether_graphite</t>
+  </si>
+  <si>
+    <t>diamond: 40 [1]</t>
+  </si>
+  <si>
+    <t>coal: 15</t>
+  </si>
+  <si>
+    <t>nether_gypsum</t>
+  </si>
+  <si>
+    <t>borax: 20 [1]</t>
+  </si>
+  <si>
+    <t>calcite: 30 [1]</t>
+  </si>
+  <si>
+    <t>nether_hematite</t>
+  </si>
+  <si>
+    <t>hematite: 35 [3]</t>
+  </si>
+  <si>
+    <t>nether_lapis</t>
+  </si>
+  <si>
+    <t>lazurite: 35 [1]</t>
+  </si>
+  <si>
+    <t>sodalite: 25 [1]</t>
+  </si>
+  <si>
+    <t>lapis: 25 [1]</t>
+  </si>
+  <si>
+    <t>nether_lubricant</t>
+  </si>
+  <si>
+    <t>soapstone: 30 [1]</t>
   </si>
   <si>
     <t>talc: 20 [1]</t>
-  </si>
-  <si>
-    <t>trona: 15</t>
-  </si>
-  <si>
-    <t>pentlandite: 5</t>
-  </si>
-  <si>
-    <t>mars_neodynium</t>
-  </si>
-  <si>
-    <t>bastnasite: 50 [1]</t>
-  </si>
-  <si>
-    <t>mars_nickel</t>
-  </si>
-  <si>
-    <t>garnierite: 25 [1]</t>
-  </si>
-  <si>
-    <t>nickel: 20</t>
-  </si>
-  <si>
-    <t>mars_pitchblende</t>
-  </si>
-  <si>
-    <t>pitchblende: 35 [1]</t>
-  </si>
-  <si>
-    <t>hematite: 25</t>
-  </si>
-  <si>
-    <t>mars_quartzite</t>
-  </si>
-  <si>
-    <t>mars_salt</t>
-  </si>
-  <si>
-    <t>rock_salt: 20 [1]</t>
-  </si>
-  <si>
-    <t>mars_stibnite</t>
-  </si>
-  <si>
-    <t>mars_sulfur</t>
-  </si>
-  <si>
-    <t>sulfur: 15</t>
-  </si>
-  <si>
-    <t>pyrite: 45</t>
-  </si>
-  <si>
-    <t>sphalerite: 25</t>
-  </si>
-  <si>
-    <t>mars_tantalite</t>
-  </si>
-  <si>
-    <t>grossular: 10</t>
-  </si>
-  <si>
-    <t>spessartine: 10</t>
-  </si>
-  <si>
-    <t>pyrolusite: 40 [1]</t>
-  </si>
-  <si>
-    <t>tantalite: 35 [1]</t>
-  </si>
-  <si>
-    <t>mars_tungsten</t>
-  </si>
-  <si>
-    <t>tungstate: 35</t>
-  </si>
-  <si>
-    <t>mars_surface_bismuthinite</t>
-  </si>
-  <si>
-    <t>bismuth: 20 [1]</t>
-  </si>
-  <si>
-    <t>sulfur: 10</t>
-  </si>
-  <si>
-    <t>gypsum: 10</t>
-  </si>
-  <si>
-    <t>mars_surface_cassiterite</t>
-  </si>
-  <si>
-    <t>cassiterite: 55 [1]</t>
-  </si>
-  <si>
-    <t>tin: 35</t>
-  </si>
-  <si>
-    <t>saltpeter: 10</t>
-  </si>
-  <si>
-    <t>mars_surface_hematite</t>
-  </si>
-  <si>
-    <t>calcite: 5</t>
-  </si>
-  <si>
-    <t>mars_surface_nickel_galena</t>
-  </si>
-  <si>
-    <t>cobaltite: 10</t>
-  </si>
-  <si>
-    <t>mars_surface_tetrahedrite</t>
-  </si>
-  <si>
-    <t>tetrahedrite: 60 [1]</t>
-  </si>
-  <si>
-    <t>redstone: 5</t>
-  </si>
-  <si>
-    <t>glacio_stone</t>
-  </si>
-  <si>
-    <t>moon_deepslate</t>
-  </si>
-  <si>
-    <t>moon_stone</t>
-  </si>
-  <si>
-    <t>moon_apatite</t>
-  </si>
-  <si>
-    <t>apatite: 25</t>
-  </si>
-  <si>
-    <t>pyrochlore: 40 [1]</t>
-  </si>
-  <si>
-    <t>olivine: 5</t>
-  </si>
-  <si>
-    <t>moon_bauxite</t>
-  </si>
-  <si>
-    <t>bauxite: 35 [1]</t>
-  </si>
-  <si>
-    <t>ilmenite: 40 [1]</t>
-  </si>
-  <si>
-    <t>armalcolite: 20</t>
-  </si>
-  <si>
-    <t>moon_beryllium</t>
-  </si>
-  <si>
-    <t>beryllium: 35 [1]</t>
-  </si>
-  <si>
-    <t>emerald: 50 [2]</t>
-  </si>
-  <si>
-    <t>thorium: 1</t>
-  </si>
-  <si>
-    <t>moon_cassiterite</t>
-  </si>
-  <si>
-    <t>chalcopyrite: 30 [1]</t>
-  </si>
-  <si>
-    <t>zeolite: 5</t>
-  </si>
-  <si>
-    <t>cassiterite: 35 [1]</t>
-  </si>
-  <si>
-    <t>tin: 15</t>
-  </si>
-  <si>
-    <t>moon_sheldonite</t>
-  </si>
-  <si>
-    <t>moon_desh</t>
-  </si>
-  <si>
-    <t>desh: 25</t>
-  </si>
-  <si>
-    <t>ilmenite: 30 [1]</t>
-  </si>
-  <si>
-    <t>aluminium: 25</t>
-  </si>
-  <si>
-    <t>moon_garnet</t>
-  </si>
-  <si>
-    <t>red_garnet: 10</t>
-  </si>
-  <si>
-    <t>yellow_garnet: 15</t>
-  </si>
-  <si>
-    <t>amethyst: 40 [1]</t>
-  </si>
-  <si>
-    <t>opal: 40 [1]</t>
-  </si>
-  <si>
-    <t>moon_garnierite</t>
-  </si>
-  <si>
-    <t>pentlandite: 25 [1]</t>
-  </si>
-  <si>
-    <t>moon_gold</t>
-  </si>
-  <si>
-    <t>magnetite: 20</t>
-  </si>
-  <si>
-    <t>moon_graphite</t>
-  </si>
-  <si>
-    <t>graphite: 50 [1]</t>
-  </si>
-  <si>
-    <t>diamond: 35</t>
-  </si>
-  <si>
-    <t>olivine: 10</t>
-  </si>
-  <si>
-    <t>moon_gypsum</t>
-  </si>
-  <si>
-    <t>calcite: 25</t>
-  </si>
-  <si>
-    <t>gypsum: 35 [1]</t>
-  </si>
-  <si>
-    <t>moon_lubricant</t>
-  </si>
-  <si>
-    <t>moon_magnetite</t>
-  </si>
-  <si>
-    <t>magnetite: 25</t>
-  </si>
-  <si>
-    <t>chromite: 40 [2]</t>
-  </si>
-  <si>
-    <t>moon_manganese</t>
-  </si>
-  <si>
-    <t>moon_mica</t>
-  </si>
-  <si>
-    <t>kyanite: 35 [1]</t>
-  </si>
-  <si>
-    <t>aluminium: 15</t>
-  </si>
-  <si>
-    <t>moon_molybdenum</t>
-  </si>
-  <si>
-    <t>moon_monazite</t>
-  </si>
-  <si>
-    <t>olivine: 1</t>
-  </si>
-  <si>
-    <t>moon_pyrolusite</t>
-  </si>
-  <si>
-    <t>pyrolusite: 40 [2]</t>
-  </si>
-  <si>
-    <t>cobaltite: 25</t>
-  </si>
-  <si>
-    <t>cobalt: 25</t>
-  </si>
-  <si>
-    <t>tantalite: 15</t>
-  </si>
-  <si>
-    <t>moon_quartz</t>
-  </si>
-  <si>
-    <t>quartzite: 20</t>
-  </si>
-  <si>
-    <t>certus_quartz: 45 [2]</t>
-  </si>
-  <si>
-    <t>nether_quartz: 30 [1]</t>
-  </si>
-  <si>
-    <t>barite: 5</t>
-  </si>
-  <si>
-    <t>moon_redstone</t>
-  </si>
-  <si>
-    <t>moon_saltpeter</t>
-  </si>
-  <si>
-    <t>saltpeter: 35 [1]</t>
-  </si>
-  <si>
-    <t>soapstone: 25</t>
-  </si>
-  <si>
-    <t>electrotine: 45</t>
-  </si>
-  <si>
-    <t>talc: 15</t>
-  </si>
-  <si>
-    <t>moon_sapphire</t>
-  </si>
-  <si>
-    <t>olivine: 2</t>
-  </si>
-  <si>
-    <t>moon_scheelite</t>
-  </si>
-  <si>
-    <t>scheelite: 40 [1]</t>
-  </si>
-  <si>
-    <t>tungstate: 50 [2]</t>
-  </si>
-  <si>
-    <t>lithium: 10</t>
-  </si>
-  <si>
-    <t>moon_silver</t>
-  </si>
-  <si>
-    <t>silver: 45 [1]</t>
-  </si>
-  <si>
-    <t>moon_sphalerite</t>
-  </si>
-  <si>
-    <t>desh: 10</t>
-  </si>
-  <si>
-    <t>sphalerite: 50 [1]</t>
-  </si>
-  <si>
-    <t>pyrite: 40</t>
-  </si>
-  <si>
-    <t>moon_tetrahedrite</t>
-  </si>
-  <si>
-    <t>tetrahedrite: 40 [1]</t>
-  </si>
-  <si>
-    <t>copper: 15</t>
-  </si>
-  <si>
-    <t>chalcocite: 25</t>
-  </si>
-  <si>
-    <t>moon_topaz</t>
-  </si>
-  <si>
-    <t>blackstone</t>
-  </si>
-  <si>
-    <t>deepslate</t>
-  </si>
-  <si>
-    <t>dripstone</t>
-  </si>
-  <si>
-    <t>nether_anthracite</t>
-  </si>
-  <si>
-    <t>anthracite: 100</t>
-  </si>
-  <si>
-    <t>nether_apatite</t>
-  </si>
-  <si>
-    <t>apatite: 50 [2]</t>
-  </si>
-  <si>
-    <t>tricalcium_phosphate: 35 [1]</t>
-  </si>
-  <si>
-    <t>nether_basaltic_sands</t>
-  </si>
-  <si>
-    <t>basaltic_mineral_sand: 35 [1]</t>
-  </si>
-  <si>
-    <t>granitic_mineral_sand: 25 [1]</t>
-  </si>
-  <si>
-    <t>fullers_earth: 25 [1]</t>
-  </si>
-  <si>
-    <t>nether_beryllium</t>
-  </si>
-  <si>
-    <t>nether_cassiterite</t>
-  </si>
-  <si>
-    <t>cassiterite: 40 [2]</t>
-  </si>
-  <si>
-    <t>tin: 60 [2]</t>
-  </si>
-  <si>
-    <t>nether_sheldonite</t>
-  </si>
-  <si>
-    <t>nether_copper</t>
-  </si>
-  <si>
-    <t>chalcopyrite: 20 [1]</t>
-  </si>
-  <si>
-    <t>pyrite: 10 [1]</t>
-  </si>
-  <si>
-    <t>copper: 65 [2]</t>
-  </si>
-  <si>
-    <t>nether_garnet</t>
-  </si>
-  <si>
-    <t>red_garnet: 10 [1]</t>
-  </si>
-  <si>
-    <t>amethyst: 40 [2]</t>
-  </si>
-  <si>
-    <t>opal: 40 [2]</t>
-  </si>
-  <si>
-    <t>nether_garnet_tin</t>
-  </si>
-  <si>
-    <t>cassiterite_sand: 35 [1]</t>
-  </si>
-  <si>
-    <t>garnet_sand: 25 [1]</t>
-  </si>
-  <si>
-    <t>asbestos: 25 [1]</t>
-  </si>
-  <si>
-    <t>nether_garnierite</t>
-  </si>
-  <si>
-    <t>cobaltite: 20 [1]</t>
-  </si>
-  <si>
-    <t>nether_goethite</t>
-  </si>
-  <si>
-    <t>goethite: 50 [3]</t>
-  </si>
-  <si>
-    <t>yellow_limonite: 15 [1]</t>
-  </si>
-  <si>
-    <t>nether_gold</t>
-  </si>
-  <si>
-    <t>nether_graphite</t>
-  </si>
-  <si>
-    <t>diamond: 40 [1]</t>
-  </si>
-  <si>
-    <t>coal: 15</t>
-  </si>
-  <si>
-    <t>nether_gypsum</t>
-  </si>
-  <si>
-    <t>borax: 20 [1]</t>
-  </si>
-  <si>
-    <t>calcite: 30 [1]</t>
-  </si>
-  <si>
-    <t>nether_hematite</t>
-  </si>
-  <si>
-    <t>hematite: 35 [3]</t>
-  </si>
-  <si>
-    <t>nether_lapis</t>
-  </si>
-  <si>
-    <t>lazurite: 35 [1]</t>
-  </si>
-  <si>
-    <t>sodalite: 25 [1]</t>
-  </si>
-  <si>
-    <t>lapis: 25 [1]</t>
-  </si>
-  <si>
-    <t>nether_lubricant</t>
-  </si>
-  <si>
-    <t>soapstone: 30 [1]</t>
   </si>
   <si>
     <t>glauconite_sand: 25 [1]</t>
@@ -6317,7 +6320,7 @@
     <col min="9" max="9" width="9.140625" customWidth="1" style="3"/>
     <col min="10" max="10" width="18.350568771362305" customWidth="1" style="3"/>
     <col min="11" max="11" width="23.763607025146484" customWidth="1" style="3"/>
-    <col min="12" max="12" width="19.039091110229492" customWidth="1" style="3"/>
+    <col min="12" max="12" width="17.945432662963867" customWidth="1" style="3"/>
     <col min="13" max="13" width="18.38944435119629" customWidth="1" style="3"/>
     <col min="14" max="14" width="13.724266052246094" customWidth="1" style="3"/>
     <col min="15" max="15" width="11.552298545837402" customWidth="1" style="3"/>
@@ -7495,13 +7498,13 @@
         <v>279</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>185</v>
+        <v>280</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O14" s="3" t="s">
         <v>115</v>
@@ -7560,7 +7563,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -7581,7 +7584,7 @@
         <v>45</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>177</v>
@@ -7646,7 +7649,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -7667,10 +7670,10 @@
         <v>55</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>126</v>
@@ -7732,7 +7735,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -7753,13 +7756,13 @@
         <v>20</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>250</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -7815,7 +7818,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -7901,7 +7904,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>38</v>
@@ -7925,7 +7928,7 @@
         <v>6</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>214</v>
@@ -7990,7 +7993,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -8076,7 +8079,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -8097,13 +8100,13 @@
         <v>45</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>131</v>
@@ -8162,7 +8165,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -8183,16 +8186,16 @@
         <v>42</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -8248,7 +8251,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -8272,7 +8275,7 @@
         <v>81</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>83</v>
@@ -8334,7 +8337,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -8355,16 +8358,16 @@
         <v>45</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>275</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>35</v>
@@ -8420,7 +8423,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -8441,13 +8444,13 @@
         <v>45</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -8503,7 +8506,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -8533,7 +8536,7 @@
         <v>55</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>35</v>
@@ -8589,7 +8592,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -8613,7 +8616,7 @@
         <v>219</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>205</v>
@@ -8622,7 +8625,7 @@
         <v>107</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>35</v>
@@ -8678,7 +8681,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -8699,7 +8702,7 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>243</v>
@@ -8708,7 +8711,7 @@
         <v>223</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -8867,16 +8870,16 @@
         <v>19</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="Y1" s="4" t="s">
         <v>26</v>
@@ -8884,7 +8887,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -8905,16 +8908,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -8949,7 +8952,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -8970,13 +8973,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>35</v>
@@ -9011,7 +9014,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>99</v>
@@ -9035,16 +9038,16 @@
         <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>213</v>
@@ -9082,7 +9085,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>31</v>
@@ -9103,16 +9106,16 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>35</v>
@@ -9147,7 +9150,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -9212,7 +9215,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -9233,16 +9236,16 @@
         <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -9277,7 +9280,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>38</v>
@@ -9301,16 +9304,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -9345,7 +9348,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -9366,16 +9369,16 @@
         <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>126</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>128</v>
@@ -9413,7 +9416,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>38</v>
@@ -9443,7 +9446,7 @@
         <v>269</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>132</v>
@@ -9481,7 +9484,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>99</v>
@@ -9505,13 +9508,13 @@
         <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>35</v>
@@ -9546,7 +9549,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -9573,16 +9576,16 @@
         <v>138</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>203</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>35</v>
@@ -9617,7 +9620,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -9685,7 +9688,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -9706,13 +9709,13 @@
         <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>63</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>65</v>
@@ -9753,7 +9756,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -9818,7 +9821,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -9839,7 +9842,7 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>172</v>
@@ -9848,10 +9851,10 @@
         <v>173</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>35</v>
@@ -9886,7 +9889,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -9916,7 +9919,7 @@
         <v>70</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -9951,7 +9954,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -9972,7 +9975,7 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>177</v>
@@ -9981,7 +9984,7 @@
         <v>178</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="P18" s="1" t="s">
         <v>36</v>
@@ -10016,7 +10019,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -10037,16 +10040,16 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>36</v>
@@ -10081,7 +10084,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -10102,16 +10105,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -10146,7 +10149,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -10176,7 +10179,7 @@
         <v>193</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>36</v>
@@ -10211,7 +10214,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -10232,16 +10235,16 @@
         <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>387</v>
+        <v>279</v>
       </c>
       <c r="P22" s="1" t="s">
         <v>36</v>
@@ -10439,7 +10442,7 @@
         <v>266</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -10990,13 +10993,13 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>213</v>
@@ -11117,7 +11120,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -11359,16 +11362,16 @@
         <v>45</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>435</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>128</v>
@@ -11622,7 +11625,7 @@
         <v>140</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>35</v>
@@ -11805,13 +11808,13 @@
         <v>453</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>279</v>
+        <v>454</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>159</v>
@@ -11846,7 +11849,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -11867,16 +11870,16 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>164</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>66</v>
@@ -11911,7 +11914,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -11932,13 +11935,13 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>169</v>
@@ -11973,7 +11976,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -11994,13 +11997,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>35</v>
@@ -12032,7 +12035,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -12059,10 +12062,10 @@
         <v>69</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -12094,7 +12097,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -12115,13 +12118,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -12153,7 +12156,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -12174,7 +12177,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>36</v>
@@ -12206,7 +12209,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -12227,13 +12230,13 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>185</v>
@@ -12268,7 +12271,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -12327,7 +12330,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -12348,13 +12351,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -12386,7 +12389,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -12410,10 +12413,10 @@
         <v>191</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -12445,7 +12448,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -12466,13 +12469,13 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>203</v>
@@ -12507,7 +12510,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
@@ -12537,10 +12540,10 @@
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>35</v>
@@ -12572,7 +12575,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -12593,13 +12596,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>82</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>35</v>
@@ -12631,7 +12634,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -12655,10 +12658,10 @@
         <v>265</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>35</v>
@@ -12690,7 +12693,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -12711,13 +12714,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>210</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>36</v>
@@ -12749,7 +12752,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -12770,13 +12773,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>36</v>
@@ -12808,7 +12811,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -12829,7 +12832,7 @@
         <v>17</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>35</v>
@@ -12861,7 +12864,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -12882,10 +12885,10 @@
         <v>45</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>223</v>
@@ -12920,7 +12923,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
added extra info to EMI ore vein tab
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -680,10 +680,10 @@
     <t>normal_tarkianite</t>
   </si>
   <si>
+    <t>tarkianite: 35</t>
+  </si>
+  <si>
     <t>oilsands: 35</t>
-  </si>
-  <si>
-    <t>tarkianite: 35</t>
   </si>
   <si>
     <t>normal_tetrahedrite</t>
@@ -5758,7 +5758,7 @@
         <v>99</v>
       </c>
       <c r="C44" s="3">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D44" s="3">
         <v>0.35</v>

</xml_diff>

<commit_message>
added saltpeter to cassiterite veins
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="514">
   <si>
     <t>Vein ID</t>
   </si>
@@ -344,10 +344,13 @@
     <t>normal_cassiterite</t>
   </si>
   <si>
-    <t>cassiterite: 40 [1]</t>
-  </si>
-  <si>
-    <t>tin: 60 [1]</t>
+    <t>cassiterite: 35 [1]</t>
+  </si>
+  <si>
+    <t>tin: 55 [1]</t>
+  </si>
+  <si>
+    <t>saltpeter: 10</t>
   </si>
   <si>
     <t>normal_coal</t>
@@ -713,10 +716,10 @@
     <t>surface_cassiterite</t>
   </si>
   <si>
-    <t>cassiterite: 60</t>
-  </si>
-  <si>
-    <t>tin: 40</t>
+    <t>cassiterite: 55</t>
+  </si>
+  <si>
+    <t>tin: 35</t>
   </si>
   <si>
     <t>surface_copper</t>
@@ -959,12 +962,6 @@
     <t>cassiterite: 55 [1]</t>
   </si>
   <si>
-    <t>tin: 35</t>
-  </si>
-  <si>
-    <t>saltpeter: 10</t>
-  </si>
-  <si>
     <t>mars_surface_hematite</t>
   </si>
   <si>
@@ -1038,9 +1035,6 @@
   </si>
   <si>
     <t>zeolite: 5</t>
-  </si>
-  <si>
-    <t>cassiterite: 35 [1]</t>
   </si>
   <si>
     <t>tin: 15</t>
@@ -3332,6 +3326,9 @@
       <c r="K18" s="3" t="s">
         <v>110</v>
       </c>
+      <c r="L18" s="3" t="s">
+        <v>111</v>
+      </c>
       <c r="P18" s="2" t="s">
         <v>35</v>
       </c>
@@ -3395,7 +3392,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -3416,7 +3413,7 @@
         <v>60</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P19" s="2" t="s">
         <v>35</v>
@@ -3481,7 +3478,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -3502,16 +3499,16 @@
         <v>40</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -3576,7 +3573,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -3597,16 +3594,16 @@
         <v>40</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>36</v>
@@ -3671,7 +3668,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -3692,19 +3689,19 @@
         <v>40</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -3769,7 +3766,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
@@ -3796,13 +3793,13 @@
         <v>47</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P23" s="1" t="s">
         <v>36</v>
@@ -3867,7 +3864,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>38</v>
@@ -3891,13 +3888,13 @@
         <v>6</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>36</v>
@@ -3962,7 +3959,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>38</v>
@@ -3986,16 +3983,16 @@
         <v>9</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -4060,7 +4057,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -4081,13 +4078,13 @@
         <v>40</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>55</v>
@@ -4155,7 +4152,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -4176,16 +4173,16 @@
         <v>40</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>35</v>
@@ -4250,7 +4247,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -4271,16 +4268,16 @@
         <v>40</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -4345,7 +4342,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -4366,19 +4363,19 @@
         <v>36</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>35</v>
@@ -4443,7 +4440,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>31</v>
@@ -4464,16 +4461,16 @@
         <v>30</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>35</v>
@@ -4538,7 +4535,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -4559,16 +4556,16 @@
         <v>30</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P31" s="1" t="s">
         <v>36</v>
@@ -4633,7 +4630,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -4654,16 +4651,16 @@
         <v>36</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>35</v>
@@ -4728,7 +4725,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -4749,13 +4746,13 @@
         <v>35</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="P33" s="2" t="s">
         <v>35</v>
@@ -4820,7 +4817,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -4841,7 +4838,7 @@
         <v>55</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P34" s="2" t="s">
         <v>35</v>
@@ -4906,7 +4903,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -4927,16 +4924,16 @@
         <v>26</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P35" s="1" t="s">
         <v>36</v>
@@ -5001,7 +4998,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -5022,13 +5019,13 @@
         <v>40</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P36" s="2" t="s">
         <v>35</v>
@@ -5093,7 +5090,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>31</v>
@@ -5114,13 +5111,13 @@
         <v>40</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P37" s="2" t="s">
         <v>35</v>
@@ -5185,7 +5182,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>38</v>
@@ -5209,16 +5206,16 @@
         <v>4</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P38" s="2" t="s">
         <v>35</v>
@@ -5283,7 +5280,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>31</v>
@@ -5304,16 +5301,16 @@
         <v>40</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>35</v>
@@ -5378,7 +5375,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>31</v>
@@ -5399,13 +5396,13 @@
         <v>40</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P40" s="2" t="s">
         <v>35</v>
@@ -5470,7 +5467,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>31</v>
@@ -5491,13 +5488,13 @@
         <v>40</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="P41" s="1" t="s">
         <v>36</v>
@@ -5562,7 +5559,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>38</v>
@@ -5586,16 +5583,16 @@
         <v>6</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P42" s="2" t="s">
         <v>35</v>
@@ -5660,7 +5657,7 @@
     </row>
     <row r="43">
       <c r="A43" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>31</v>
@@ -5681,13 +5678,13 @@
         <v>45</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P43" s="1" t="s">
         <v>36</v>
@@ -5752,7 +5749,7 @@
     </row>
     <row r="44">
       <c r="A44" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>99</v>
@@ -5776,16 +5773,16 @@
         <v>10</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P44" s="1" t="s">
         <v>36</v>
@@ -5850,7 +5847,7 @@
     </row>
     <row r="45">
       <c r="A45" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>31</v>
@@ -5871,13 +5868,13 @@
         <v>40</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P45" s="2" t="s">
         <v>35</v>
@@ -5942,7 +5939,7 @@
     </row>
     <row r="46">
       <c r="A46" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>31</v>
@@ -5963,13 +5960,13 @@
         <v>50</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K46" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="L46" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>107</v>
@@ -6037,7 +6034,7 @@
     </row>
     <row r="47">
       <c r="A47" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>31</v>
@@ -6058,10 +6055,13 @@
         <v>50</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
+      </c>
+      <c r="L47" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="P47" s="2" t="s">
         <v>35</v>
@@ -6126,7 +6126,7 @@
     </row>
     <row r="48">
       <c r="A48" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>31</v>
@@ -6147,16 +6147,16 @@
         <v>50</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L48" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M48" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P48" s="1" t="s">
         <v>36</v>
@@ -6221,7 +6221,7 @@
     </row>
     <row r="49">
       <c r="A49" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>31</v>
@@ -6242,13 +6242,13 @@
         <v>50</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P49" s="1" t="s">
         <v>36</v>
@@ -6313,7 +6313,7 @@
     </row>
     <row r="50">
       <c r="A50" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>31</v>
@@ -6334,13 +6334,13 @@
         <v>50</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L50" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P50" s="2" t="s">
         <v>35</v>
@@ -6529,10 +6529,10 @@
         <v>22</v>
       </c>
       <c r="AB1" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AC1" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AD1" s="4" t="s">
         <v>26</v>
@@ -6541,12 +6541,12 @@
         <v>28</v>
       </c>
       <c r="AF1" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -6567,13 +6567,13 @@
         <v>60</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -6629,7 +6629,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -6653,7 +6653,7 @@
         <v>72</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>73</v>
@@ -6712,7 +6712,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>31</v>
@@ -6736,13 +6736,13 @@
         <v>32</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>35</v>
@@ -6798,7 +6798,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>38</v>
@@ -6825,7 +6825,7 @@
         <v>76</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>78</v>
@@ -6834,7 +6834,7 @@
         <v>79</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>35</v>
@@ -6890,7 +6890,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -6920,7 +6920,7 @@
         <v>92</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>35</v>
@@ -6976,7 +6976,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>99</v>
@@ -7006,7 +7006,7 @@
         <v>101</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -7062,7 +7062,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -7083,10 +7083,10 @@
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P8" s="2" t="s">
         <v>35</v>
@@ -7142,7 +7142,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -7163,16 +7163,16 @@
         <v>50</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L9" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>35</v>
@@ -7228,7 +7228,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -7249,16 +7249,16 @@
         <v>50</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>35</v>
@@ -7314,7 +7314,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -7335,16 +7335,16 @@
         <v>40</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>35</v>
@@ -7400,7 +7400,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>99</v>
@@ -7424,16 +7424,16 @@
         <v>9</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>35</v>
@@ -7489,7 +7489,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -7510,13 +7510,13 @@
         <v>40</v>
       </c>
       <c r="J13" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="K13" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="L13" s="3" t="s">
         <v>144</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>143</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>55</v>
@@ -7575,7 +7575,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -7596,22 +7596,22 @@
         <v>40</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>35</v>
@@ -7667,7 +7667,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -7688,16 +7688,16 @@
         <v>45</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>35</v>
@@ -7753,7 +7753,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -7774,16 +7774,16 @@
         <v>55</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>35</v>
@@ -7839,7 +7839,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -7860,13 +7860,13 @@
         <v>20</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -7922,7 +7922,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -7943,16 +7943,16 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>35</v>
@@ -8008,7 +8008,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>38</v>
@@ -8032,16 +8032,16 @@
         <v>6</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P19" s="2" t="s">
         <v>35</v>
@@ -8097,7 +8097,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -8118,16 +8118,16 @@
         <v>40</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>35</v>
@@ -8183,7 +8183,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -8204,16 +8204,16 @@
         <v>45</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>35</v>
@@ -8269,7 +8269,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -8290,16 +8290,16 @@
         <v>42</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -8355,7 +8355,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -8379,13 +8379,13 @@
         <v>81</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>83</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -8441,7 +8441,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -8462,16 +8462,16 @@
         <v>45</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>35</v>
@@ -8527,7 +8527,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -8548,13 +8548,13 @@
         <v>45</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>314</v>
+        <v>234</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>315</v>
+        <v>111</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -8610,7 +8610,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -8631,16 +8631,16 @@
         <v>45</v>
       </c>
       <c r="J26" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="K26" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>144</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>55</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>35</v>
@@ -8696,7 +8696,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -8717,19 +8717,19 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>107</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>35</v>
@@ -8785,7 +8785,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -8806,16 +8806,16 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="M28" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="M28" s="3" t="s">
-        <v>322</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -8974,16 +8974,16 @@
         <v>19</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="X1" s="4" t="s">
         <v>324</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>325</v>
       </c>
       <c r="Y1" s="4" t="s">
         <v>26</v>
@@ -8991,7 +8991,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -9012,16 +9012,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>328</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>329</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -9056,7 +9056,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -9077,13 +9077,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>332</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>333</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>35</v>
@@ -9118,7 +9118,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>99</v>
@@ -9142,19 +9142,19 @@
         <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>337</v>
-      </c>
       <c r="M4" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>35</v>
@@ -9189,7 +9189,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>31</v>
@@ -9210,16 +9210,16 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="M5" s="3" t="s">
         <v>340</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>342</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>35</v>
@@ -9254,7 +9254,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -9278,13 +9278,13 @@
         <v>32</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L6" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="M6" s="3" t="s">
         <v>256</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>36</v>
@@ -9319,7 +9319,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -9340,16 +9340,16 @@
         <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>347</v>
-      </c>
       <c r="M7" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -9384,7 +9384,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>38</v>
@@ -9408,16 +9408,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="M8" s="3" t="s">
         <v>350</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>352</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -9452,7 +9452,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -9473,19 +9473,19 @@
         <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>35</v>
@@ -9520,7 +9520,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>38</v>
@@ -9544,16 +9544,16 @@
         <v>10</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>35</v>
@@ -9588,7 +9588,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>99</v>
@@ -9612,13 +9612,13 @@
         <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <v>358</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>360</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>35</v>
@@ -9653,7 +9653,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -9677,19 +9677,19 @@
         <v>9</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>35</v>
@@ -9724,7 +9724,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -9745,19 +9745,19 @@
         <v>30</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P13" s="2" t="s">
         <v>35</v>
@@ -9792,7 +9792,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -9813,13 +9813,13 @@
         <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>63</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>65</v>
@@ -9860,7 +9860,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -9881,16 +9881,16 @@
         <v>30</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>36</v>
@@ -9925,7 +9925,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -9946,19 +9946,19 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>35</v>
@@ -9993,7 +9993,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -10023,7 +10023,7 @@
         <v>70</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -10058,7 +10058,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -10079,16 +10079,16 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="P18" s="1" t="s">
         <v>36</v>
@@ -10123,7 +10123,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -10144,16 +10144,16 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="L19" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="M19" s="3" t="s">
         <v>377</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>379</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>36</v>
@@ -10188,7 +10188,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -10209,16 +10209,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="M20" s="3" t="s">
         <v>382</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>384</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -10253,7 +10253,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -10274,16 +10274,16 @@
         <v>35</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>36</v>
@@ -10318,7 +10318,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -10339,16 +10339,16 @@
         <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="K22" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>389</v>
-      </c>
       <c r="M22" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P22" s="1" t="s">
         <v>36</v>
@@ -10383,7 +10383,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
@@ -10410,7 +10410,7 @@
         <v>76</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>78</v>
@@ -10419,7 +10419,7 @@
         <v>79</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -10454,7 +10454,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -10475,13 +10475,13 @@
         <v>20</v>
       </c>
       <c r="J24" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>393</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>395</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>35</v>
@@ -10516,7 +10516,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -10537,16 +10537,16 @@
         <v>30</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -10581,7 +10581,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -10602,13 +10602,13 @@
         <v>35</v>
       </c>
       <c r="J26" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="L26" s="3" t="s">
         <v>399</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="L26" s="3" t="s">
-        <v>401</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>36</v>
@@ -10643,7 +10643,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -10664,16 +10664,16 @@
         <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="M27" s="3" t="s">
         <v>403</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="M27" s="3" t="s">
-        <v>405</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -10708,7 +10708,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
@@ -10867,16 +10867,16 @@
         <v>11</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>19</v>
@@ -10893,7 +10893,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -10917,7 +10917,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -10949,7 +10949,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -10970,10 +10970,10 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>92</v>
@@ -11008,7 +11008,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -11032,13 +11032,13 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>416</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>418</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>97</v>
@@ -11073,7 +11073,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>99</v>
@@ -11097,16 +11097,16 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="L5" s="3" t="s">
-        <v>337</v>
-      </c>
       <c r="M5" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>36</v>
@@ -11138,7 +11138,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -11159,10 +11159,13 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>422</v>
+        <v>420</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>35</v>
@@ -11194,7 +11197,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -11224,7 +11227,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -11256,7 +11259,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -11277,16 +11280,16 @@
         <v>45</v>
       </c>
       <c r="J8" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="M8" s="3" t="s">
         <v>425</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>426</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>427</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -11318,7 +11321,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>38</v>
@@ -11342,16 +11345,16 @@
         <v>8</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>36</v>
@@ -11383,7 +11386,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -11404,16 +11407,16 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="L10" s="3" t="s">
         <v>433</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>434</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>435</v>
-      </c>
       <c r="M10" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>35</v>
@@ -11445,7 +11448,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -11466,19 +11469,19 @@
         <v>45</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>35</v>
@@ -11510,7 +11513,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>31</v>
@@ -11531,10 +11534,10 @@
         <v>37</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>49</v>
@@ -11572,7 +11575,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -11634,7 +11637,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>99</v>
@@ -11658,13 +11661,13 @@
         <v>12</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>35</v>
@@ -11696,7 +11699,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
@@ -11720,16 +11723,16 @@
         <v>9</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>35</v>
@@ -11761,7 +11764,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -11788,7 +11791,7 @@
         <v>53</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>55</v>
@@ -11826,7 +11829,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -11847,16 +11850,16 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="L17" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="K17" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>453</v>
-      </c>
       <c r="M17" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -11888,7 +11891,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -11909,19 +11912,19 @@
         <v>41</v>
       </c>
       <c r="J18" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="M18" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="L18" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>458</v>
-      </c>
       <c r="N18" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>35</v>
@@ -11953,7 +11956,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -11974,16 +11977,16 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="M19" s="3" t="s">
         <v>460</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>462</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>66</v>
@@ -12018,7 +12021,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -12039,16 +12042,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="K20" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>466</v>
-      </c>
       <c r="M20" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -12080,7 +12083,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -12101,13 +12104,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>35</v>
@@ -12139,7 +12142,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -12166,10 +12169,10 @@
         <v>69</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -12201,7 +12204,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -12222,13 +12225,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>474</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>476</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -12260,7 +12263,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -12281,7 +12284,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>36</v>
@@ -12313,7 +12316,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -12334,16 +12337,16 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>480</v>
       </c>
-      <c r="K25" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>482</v>
-      </c>
       <c r="M25" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P25" s="1" t="s">
         <v>36</v>
@@ -12375,7 +12378,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -12434,7 +12437,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -12455,13 +12458,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="L27" s="3" t="s">
         <v>485</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>487</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -12493,7 +12496,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -12514,13 +12517,13 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -12552,7 +12555,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -12573,16 +12576,16 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>35</v>
@@ -12614,7 +12617,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
@@ -12644,10 +12647,10 @@
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>35</v>
@@ -12679,7 +12682,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -12700,13 +12703,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>82</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>35</v>
@@ -12738,7 +12741,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -12759,13 +12762,13 @@
         <v>45</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>35</v>
@@ -12797,7 +12800,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -12818,13 +12821,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>36</v>
@@ -12856,7 +12859,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -12877,13 +12880,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="L34" s="3" t="s">
         <v>507</v>
-      </c>
-      <c r="K34" s="3" t="s">
-        <v>508</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>509</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>36</v>
@@ -12915,7 +12918,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -12936,7 +12939,7 @@
         <v>17</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>35</v>
@@ -12968,7 +12971,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -12989,13 +12992,13 @@
         <v>45</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P36" s="2" t="s">
         <v>35</v>
@@ -13027,7 +13030,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
make these two venus veins more common
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="523">
   <si>
     <t>Vein ID</t>
   </si>
@@ -1563,16 +1563,28 @@
     <t>venus_manual_salt</t>
   </si>
   <si>
-    <t>salt: 50</t>
-  </si>
-  <si>
-    <t>spodumene: 15</t>
+    <t>salt: 80</t>
+  </si>
+  <si>
+    <t>rock_salt: 10</t>
+  </si>
+  <si>
+    <t>lepidolite: 5</t>
+  </si>
+  <si>
+    <t>spodumene: 5</t>
   </si>
   <si>
     <t>venus_manual_sulfur</t>
   </si>
   <si>
-    <t>sulfur: 50</t>
+    <t>sulfur: 80</t>
+  </si>
+  <si>
+    <t>pyrite: 15</t>
+  </si>
+  <si>
+    <t>sphalerite: 5</t>
   </si>
 </sst>
 </file>
@@ -13130,8 +13142,8 @@
     <col min="9" max="9" width="9.140625" customWidth="1" style="3"/>
     <col min="10" max="10" width="9.682135581970215" customWidth="1" style="3"/>
     <col min="11" max="11" width="12.619355201721191" customWidth="1" style="3"/>
-    <col min="12" max="12" width="13.423484802246094" customWidth="1" style="3"/>
-    <col min="13" max="13" width="15.053228378295898" customWidth="1" style="3"/>
+    <col min="12" max="12" width="12.329827308654785" customWidth="1" style="3"/>
+    <col min="13" max="13" width="13.95957088470459" customWidth="1" style="3"/>
     <col min="14" max="14" width="9.140625" customWidth="1" style="3"/>
     <col min="15" max="15" width="9.140625" customWidth="1" style="3"/>
     <col min="16" max="16" width="9.140625" customWidth="1" style="3"/>
@@ -13225,7 +13237,7 @@
         <v>38</v>
       </c>
       <c r="C2" s="3">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3">
         <v>0.2</v>
@@ -13246,13 +13258,13 @@
         <v>515</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>214</v>
+        <v>516</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>198</v>
+        <v>517</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>36</v>
@@ -13275,13 +13287,13 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="3">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3">
         <v>0.2</v>
@@ -13293,16 +13305,16 @@
         <v>65</v>
       </c>
       <c r="G3" s="3">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>219</v>
+        <v>521</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>220</v>
+        <v>522</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
add tooltips to ore pages, fix density rounding, fix radioactive hazard
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="522">
   <si>
     <t>Vein ID</t>
   </si>
@@ -1543,12 +1543,6 @@
   </si>
   <si>
     <t>sphalerite: 15 [1]</t>
-  </si>
-  <si>
-    <t>nether_sylvite</t>
-  </si>
-  <si>
-    <t>sylvite: 100</t>
   </si>
   <si>
     <t>nether_tetrahedrite</t>
@@ -10898,7 +10892,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:X37"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.112842559814453" customWidth="1" style="3"/>
@@ -13041,84 +13035,96 @@
         <v>31</v>
       </c>
       <c r="C35" s="3">
-        <v>75</v>
+        <v>170</v>
       </c>
       <c r="D35" s="3">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E35" s="3">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F35" s="3">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="G35" s="3">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>510</v>
       </c>
+      <c r="K35" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>227</v>
+      </c>
       <c r="P35" s="2" t="s">
         <v>35</v>
       </c>
       <c r="Q35" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="R35" s="2" t="s">
-        <v>35</v>
+      <c r="R35" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="S35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="T35" s="2" t="s">
-        <v>35</v>
+      <c r="T35" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="U35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V35" s="2" t="s">
-        <v>35</v>
+      <c r="V35" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="W35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X35" s="2" t="s">
-        <v>35</v>
+      <c r="X35" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C36" s="3">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="D36" s="3">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E36" s="3">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F36" s="3">
         <v>128</v>
       </c>
       <c r="G36" s="3">
-        <v>45</v>
+        <v>33</v>
+      </c>
+      <c r="H36" s="3">
+        <v>7</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>512</v>
+        <v>85</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>513</v>
+        <v>86</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="P36" s="2" t="s">
-        <v>35</v>
+        <v>87</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="Q36" s="1" t="s">
         <v>36</v>
@@ -13135,78 +13141,13 @@
       <c r="U36" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V36" s="1" t="s">
-        <v>36</v>
+      <c r="V36" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="W36" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X36" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="s">
-        <v>514</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" s="3">
-        <v>180</v>
-      </c>
-      <c r="D37" s="3">
-        <v>0.4</v>
-      </c>
-      <c r="E37" s="3">
-        <v>0</v>
-      </c>
-      <c r="F37" s="3">
-        <v>128</v>
-      </c>
-      <c r="G37" s="3">
-        <v>33</v>
-      </c>
-      <c r="H37" s="3">
-        <v>7</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K37" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="M37" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="P37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="U37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="V37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="W37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X37" s="2" t="s">
+      <c r="X36" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -13320,7 +13261,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -13344,16 +13285,16 @@
         <v>6</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>516</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>517</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>518</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>519</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>36</v>
@@ -13376,7 +13317,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -13397,13 +13338,13 @@
         <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>521</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>522</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>523</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
add quartzite to mars
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -6524,7 +6524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AF29"/>
+  <dimension ref="A1:AG29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.277278900146484" customWidth="1" style="3"/>
@@ -6555,11 +6555,11 @@
     <col min="26" max="26" width="9.140625" customWidth="1" style="3"/>
     <col min="27" max="27" width="10.328712463378906" customWidth="1" style="3"/>
     <col min="28" max="28" width="11.9512939453125" customWidth="1" style="3"/>
-    <col min="29" max="29" width="11.877633094787598" customWidth="1" style="3"/>
-    <col min="30" max="30" width="9.140625" customWidth="1" style="3"/>
+    <col min="29" max="29" width="9.530721664428711" customWidth="1" style="3"/>
+    <col min="30" max="30" width="11.877633094787598" customWidth="1" style="3"/>
     <col min="31" max="31" width="9.140625" customWidth="1" style="3"/>
-    <col min="32" max="32" width="12.787137985229492" customWidth="1" style="3"/>
-    <col min="33" max="33" width="9.140625" customWidth="1" style="3"/>
+    <col min="32" max="32" width="9.140625" customWidth="1" style="3"/>
+    <col min="33" max="33" width="12.787137985229492" customWidth="1" style="3"/>
     <col min="34" max="34" width="9.140625" customWidth="1" style="3"/>
     <col min="35" max="35" width="9.140625" customWidth="1" style="3"/>
     <col min="36" max="36" width="9.140625" customWidth="1" style="3"/>
@@ -6646,15 +6646,18 @@
         <v>248</v>
       </c>
       <c r="AC1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AD1" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="AD1" s="4" t="s">
+      <c r="AE1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AF1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AG1" s="4" t="s">
         <v>250</v>
       </c>
     </row>
@@ -6672,7 +6675,7 @@
         <v>0.3</v>
       </c>
       <c r="E2" s="3">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="F2" s="3">
         <v>0</v>
@@ -6692,52 +6695,55 @@
       <c r="P2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>36</v>
+      <c r="Q2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>35</v>
+      <c r="V2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Y2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>36</v>
+      <c r="Y2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AC2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>36</v>
+      <c r="AD2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG2" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -6755,7 +6761,7 @@
         <v>0.3</v>
       </c>
       <c r="E3" s="3">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="F3" s="3">
         <v>0</v>
@@ -6784,14 +6790,14 @@
       <c r="S3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="T3" s="1" t="s">
-        <v>36</v>
+      <c r="T3" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="U3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V3" s="1" t="s">
-        <v>36</v>
+      <c r="V3" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="W3" s="1" t="s">
         <v>36</v>
@@ -6802,26 +6808,29 @@
       <c r="Y3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="2" t="s">
-        <v>35</v>
+      <c r="Z3" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AA3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AB3" s="1" t="s">
-        <v>36</v>
+      <c r="AB3" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AC3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AD3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF3" s="1" t="s">
-        <v>36</v>
+      <c r="AD3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG3" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -6838,7 +6847,7 @@
         <v>0.3</v>
       </c>
       <c r="E4" s="3">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="F4" s="3">
         <v>0</v>
@@ -6861,23 +6870,23 @@
       <c r="P4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>36</v>
+      <c r="Q4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="T4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="U4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>36</v>
+      <c r="U4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="W4" s="1" t="s">
         <v>36</v>
@@ -6885,29 +6894,32 @@
       <c r="X4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Y4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z4" s="2" t="s">
-        <v>35</v>
+      <c r="Y4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AA4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AB4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AC4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD4" s="2" t="s">
-        <v>35</v>
+      <c r="AB4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD4" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AE4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AF4" s="1" t="s">
-        <v>36</v>
+      <c r="AF4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG4" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -6989,16 +7001,19 @@
       <c r="AB5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE5" s="1" t="s">
-        <v>36</v>
+      <c r="AC5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE5" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG5" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7075,16 +7090,19 @@
       <c r="AB6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AC6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE6" s="1" t="s">
-        <v>36</v>
+      <c r="AC6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE6" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG6" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7164,13 +7182,16 @@
       <c r="AC7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AD7" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE7" s="2" t="s">
-        <v>35</v>
+      <c r="AD7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AF7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG7" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7241,16 +7262,19 @@
       <c r="AB8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD8" s="2" t="s">
-        <v>35</v>
+      <c r="AC8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD8" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AE8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AF8" s="1" t="s">
+      <c r="AF8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG8" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7327,16 +7351,19 @@
       <c r="AB9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC9" s="2" t="s">
-        <v>35</v>
+      <c r="AC9" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AD9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE9" s="1" t="s">
-        <v>36</v>
+      <c r="AE9" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG9" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7413,16 +7440,19 @@
       <c r="AB10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF10" s="2" t="s">
+      <c r="AC10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG10" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7505,10 +7535,13 @@
       <c r="AD11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF11" s="2" t="s">
+      <c r="AE11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG11" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7588,16 +7621,19 @@
       <c r="AB12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD12" s="2" t="s">
-        <v>35</v>
+      <c r="AC12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD12" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AE12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AF12" s="1" t="s">
+      <c r="AF12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG12" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7677,13 +7713,16 @@
       <c r="AC13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD13" s="2" t="s">
-        <v>35</v>
+      <c r="AD13" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AE13" s="2" t="s">
         <v>35</v>
       </c>
       <c r="AF13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG13" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7766,10 +7805,13 @@
       <c r="AD14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF14" s="2" t="s">
+      <c r="AE14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG14" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7855,13 +7897,16 @@
       <c r="AC15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF15" s="2" t="s">
+      <c r="AD15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG15" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7938,8 +7983,8 @@
       <c r="AB16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC16" s="2" t="s">
-        <v>35</v>
+      <c r="AC16" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AD16" s="2" t="s">
         <v>35</v>
@@ -7947,7 +7992,10 @@
       <c r="AE16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AF16" s="1" t="s">
+      <c r="AF16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG16" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8027,13 +8075,16 @@
       <c r="AC17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF17" s="2" t="s">
+      <c r="AD17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG17" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -8110,13 +8161,16 @@
       <c r="AC18" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE18" s="1" t="s">
-        <v>36</v>
+      <c r="AD18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE18" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG18" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8196,13 +8250,16 @@
       <c r="AC19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE19" s="1" t="s">
-        <v>36</v>
+      <c r="AD19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE19" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG19" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8285,13 +8342,16 @@
       <c r="AC20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD20" s="2" t="s">
-        <v>35</v>
+      <c r="AD20" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AE20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AF20" s="1" t="s">
+      <c r="AF20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG20" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8371,13 +8431,16 @@
       <c r="AC21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD21" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE21" s="1" t="s">
-        <v>36</v>
+      <c r="AD21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE21" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8463,7 +8526,10 @@
       <c r="AE22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AF22" s="1" t="s">
+      <c r="AF22" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG22" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8540,16 +8606,19 @@
       <c r="AB23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC23" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE23" s="1" t="s">
-        <v>36</v>
+      <c r="AC23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE23" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG23" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8626,16 +8695,19 @@
       <c r="AB24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AC24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF24" s="2" t="s">
+      <c r="AC24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG24" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -8715,13 +8787,16 @@
       <c r="AC25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD25" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE25" s="1" t="s">
-        <v>36</v>
+      <c r="AD25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE25" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG25" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8798,13 +8873,16 @@
       <c r="AC26" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD26" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE26" s="1" t="s">
-        <v>36</v>
+      <c r="AD26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE26" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG26" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8884,13 +8962,16 @@
       <c r="AC27" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD27" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE27" s="1" t="s">
-        <v>36</v>
+      <c r="AD27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE27" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG27" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -8973,13 +9054,16 @@
       <c r="AC28" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE28" s="1" t="s">
-        <v>36</v>
+      <c r="AD28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE28" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG28" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -9059,13 +9143,16 @@
       <c r="AC29" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AD29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE29" s="1" t="s">
-        <v>36</v>
+      <c r="AD29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE29" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG29" s="1" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix venus sulfur indicators
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="525">
   <si>
     <t>Vein ID</t>
   </si>
@@ -1558,6 +1558,12 @@
   </si>
   <si>
     <t>nether_topaz</t>
+  </si>
+  <si>
+    <t>flavolite</t>
+  </si>
+  <si>
+    <t>sandy_jadestone</t>
   </si>
   <si>
     <t>venus_manual_salt</t>
@@ -1707,8 +1713,7 @@
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
     <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
     <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
-    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
-    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -6577,8 +6582,7 @@
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
     <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
     <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
-    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
-    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -9219,8 +9223,7 @@
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
     <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
     <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
-    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
-    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -11127,8 +11130,7 @@
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
     <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
     <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
-    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
-    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -13346,7 +13348,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.293367385864258" customWidth="1" style="3"/>
@@ -13369,9 +13371,9 @@
     <col min="18" max="18" width="9.140625" customWidth="1" style="3"/>
     <col min="19" max="19" width="10.040207862854004" customWidth="1" style="3"/>
     <col min="20" max="20" width="9.140625" customWidth="1" style="3"/>
-    <col min="21" max="21" width="12.787137985229492" customWidth="1" style="3"/>
-    <col min="22" max="22" width="9.140625" customWidth="1" style="3"/>
-    <col min="23" max="23" width="9.140625" customWidth="1" style="3"/>
+    <col min="21" max="21" width="9.140625" customWidth="1" style="3"/>
+    <col min="22" max="22" width="16.62772560119629" customWidth="1" style="3"/>
+    <col min="23" max="23" width="12.787137985229492" customWidth="1" style="3"/>
     <col min="24" max="24" width="9.140625" customWidth="1" style="3"/>
     <col min="25" max="25" width="9.140625" customWidth="1" style="3"/>
     <col min="26" max="26" width="9.140625" customWidth="1" style="3"/>
@@ -13396,8 +13398,7 @@
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
     <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
     <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
-    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
-    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -13444,15 +13445,21 @@
         <v>409</v>
       </c>
       <c r="T1" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="U1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="V1" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="W1" s="4" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -13476,16 +13483,16 @@
         <v>6</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>36</v>
@@ -13503,12 +13510,18 @@
         <v>36</v>
       </c>
       <c r="U2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -13529,13 +13542,13 @@
         <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>36</v>
@@ -13553,6 +13566,12 @@
         <v>36</v>
       </c>
       <c r="U3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" s="1" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
why is this sulfur vein so dense
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="619">
   <si>
     <t>Vein ID</t>
   </si>
@@ -447,7 +447,13 @@
     <t>deep_sulfur</t>
   </si>
   <si>
-    <t>sulfur: 10 [1]</t>
+    <t>sulfur: 90 [1]</t>
+  </si>
+  <si>
+    <t>bornite: 5</t>
+  </si>
+  <si>
+    <t>chalcocite: 5</t>
   </si>
   <si>
     <t>deep_tantalite</t>
@@ -510,10 +516,7 @@
     <t>high_coal</t>
   </si>
   <si>
-    <t>coal: 9</t>
-  </si>
-  <si>
-    <t>diamond: 1</t>
+    <t>coal: 100</t>
   </si>
   <si>
     <t>high_gypsum</t>
@@ -4840,7 +4843,7 @@
         <v>34</v>
       </c>
       <c r="D25" s="3">
-        <v>0.84</v>
+        <v>0.4</v>
       </c>
       <c r="E25" s="3">
         <v>-60</v>
@@ -4856,6 +4859,12 @@
       </c>
       <c r="J25" s="3" t="s">
         <v>143</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>145</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>43</v>
@@ -4944,7 +4953,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>39</v>
@@ -4965,16 +4974,16 @@
         <v>28</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>103</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>43</v>
@@ -5063,7 +5072,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>39</v>
@@ -5084,16 +5093,16 @@
         <v>28</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>43</v>
@@ -5182,7 +5191,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>39</v>
@@ -5203,10 +5212,10 @@
         <v>30</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>43</v>
@@ -5295,7 +5304,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>39</v>
@@ -5316,16 +5325,16 @@
         <v>24</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>43</v>
@@ -5414,7 +5423,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>39</v>
@@ -5435,7 +5444,7 @@
         <v>20</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P30" s="1" t="s">
         <v>44</v>
@@ -5524,7 +5533,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>39</v>
@@ -5545,10 +5554,7 @@
         <v>30</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="K31" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P31" s="1" t="s">
         <v>44</v>
@@ -5637,7 +5643,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>39</v>
@@ -5658,7 +5664,7 @@
         <v>10</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P32" s="1" t="s">
         <v>44</v>
@@ -5747,7 +5753,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>39</v>
@@ -5768,10 +5774,10 @@
         <v>20</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>44</v>
@@ -5860,7 +5866,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>46</v>
@@ -5884,13 +5890,13 @@
         <v>5</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>44</v>
@@ -5979,7 +5985,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>39</v>
@@ -6000,7 +6006,7 @@
         <v>10</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P35" s="1" t="s">
         <v>44</v>
@@ -6089,7 +6095,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>39</v>
@@ -6110,13 +6116,13 @@
         <v>25</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P36" s="1" t="s">
         <v>44</v>
@@ -6205,7 +6211,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>39</v>
@@ -6226,10 +6232,10 @@
         <v>15</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="P37" s="1" t="s">
         <v>44</v>
@@ -6318,7 +6324,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>39</v>
@@ -6339,10 +6345,10 @@
         <v>15</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P38" s="2" t="s">
         <v>43</v>
@@ -6431,7 +6437,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>39</v>
@@ -6452,10 +6458,10 @@
         <v>16</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>43</v>
@@ -6544,7 +6550,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>39</v>
@@ -6565,7 +6571,7 @@
         <v>36</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P40" s="2" t="s">
         <v>43</v>
@@ -6654,7 +6660,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>39</v>
@@ -6675,13 +6681,13 @@
         <v>20</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="P41" s="1" t="s">
         <v>44</v>
@@ -6770,7 +6776,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>39</v>
@@ -6791,10 +6797,10 @@
         <v>15</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P42" s="2" t="s">
         <v>43</v>
@@ -6883,7 +6889,7 @@
     </row>
     <row r="43">
       <c r="A43" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>39</v>
@@ -6904,13 +6910,13 @@
         <v>15</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>43</v>
@@ -6999,7 +7005,7 @@
     </row>
     <row r="44">
       <c r="A44" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>39</v>
@@ -7020,10 +7026,10 @@
         <v>15</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="P44" s="1" t="s">
         <v>44</v>
@@ -7112,7 +7118,7 @@
     </row>
     <row r="45">
       <c r="A45" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>39</v>
@@ -7133,10 +7139,10 @@
         <v>15</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P45" s="2" t="s">
         <v>43</v>
@@ -7225,7 +7231,7 @@
     </row>
     <row r="46">
       <c r="A46" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>39</v>
@@ -7246,10 +7252,10 @@
         <v>10</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K46" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="P46" s="2" t="s">
         <v>43</v>
@@ -7338,7 +7344,7 @@
     </row>
     <row r="47">
       <c r="A47" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>46</v>
@@ -7362,10 +7368,10 @@
         <v>4</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P47" s="2" t="s">
         <v>43</v>
@@ -7454,7 +7460,7 @@
     </row>
     <row r="48">
       <c r="A48" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>62</v>
@@ -7478,10 +7484,10 @@
         <v>5</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P48" s="2" t="s">
         <v>43</v>
@@ -7570,7 +7576,7 @@
     </row>
     <row r="49">
       <c r="A49" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>46</v>
@@ -7594,13 +7600,13 @@
         <v>10</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P49" s="2" t="s">
         <v>43</v>
@@ -7689,7 +7695,7 @@
     </row>
     <row r="50">
       <c r="A50" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>46</v>
@@ -7713,10 +7719,10 @@
         <v>8</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="P50" s="1" t="s">
         <v>44</v>
@@ -7805,7 +7811,7 @@
     </row>
     <row r="51">
       <c r="A51" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>62</v>
@@ -7829,13 +7835,13 @@
         <v>10</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P51" s="1" t="s">
         <v>44</v>
@@ -7924,7 +7930,7 @@
     </row>
     <row r="52">
       <c r="A52" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>39</v>
@@ -7954,7 +7960,7 @@
         <v>108</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="P52" s="2" t="s">
         <v>43</v>
@@ -8043,7 +8049,7 @@
     </row>
     <row r="53">
       <c r="A53" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>39</v>
@@ -8064,7 +8070,7 @@
         <v>15</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="P53" s="2" t="s">
         <v>43</v>
@@ -8153,7 +8159,7 @@
     </row>
     <row r="54">
       <c r="A54" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>39</v>
@@ -8174,7 +8180,7 @@
         <v>5</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="P54" s="1" t="s">
         <v>44</v>
@@ -8263,7 +8269,7 @@
     </row>
     <row r="55">
       <c r="A55" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>39</v>
@@ -8284,7 +8290,7 @@
         <v>10</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="P55" s="1" t="s">
         <v>44</v>
@@ -8373,7 +8379,7 @@
     </row>
     <row r="56">
       <c r="A56" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>39</v>
@@ -8394,7 +8400,7 @@
         <v>15</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P56" s="1" t="s">
         <v>44</v>
@@ -8483,7 +8489,7 @@
     </row>
     <row r="57">
       <c r="A57" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>39</v>
@@ -8504,7 +8510,7 @@
         <v>15</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="P57" s="2" t="s">
         <v>43</v>
@@ -8593,7 +8599,7 @@
     </row>
     <row r="58">
       <c r="A58" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>39</v>
@@ -8614,7 +8620,7 @@
         <v>15</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P58" s="2" t="s">
         <v>43</v>
@@ -8703,7 +8709,7 @@
     </row>
     <row r="59">
       <c r="A59" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>39</v>
@@ -8724,7 +8730,7 @@
         <v>15</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P59" s="2" t="s">
         <v>43</v>
@@ -8813,7 +8819,7 @@
     </row>
     <row r="60">
       <c r="A60" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>39</v>
@@ -8834,7 +8840,7 @@
         <v>5</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="P60" s="1" t="s">
         <v>44</v>
@@ -8923,7 +8929,7 @@
     </row>
     <row r="61">
       <c r="A61" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>39</v>
@@ -8944,7 +8950,7 @@
         <v>15</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P61" s="1" t="s">
         <v>44</v>
@@ -9033,7 +9039,7 @@
     </row>
     <row r="62">
       <c r="A62" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>39</v>
@@ -9054,7 +9060,7 @@
         <v>15</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P62" s="2" t="s">
         <v>43</v>
@@ -9143,7 +9149,7 @@
     </row>
     <row r="63">
       <c r="A63" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>39</v>
@@ -9164,7 +9170,7 @@
         <v>5</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="P63" s="1" t="s">
         <v>44</v>
@@ -9253,7 +9259,7 @@
     </row>
     <row r="64">
       <c r="A64" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>39</v>
@@ -9274,7 +9280,7 @@
         <v>15</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P64" s="1" t="s">
         <v>44</v>
@@ -9363,7 +9369,7 @@
     </row>
     <row r="65">
       <c r="A65" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>39</v>
@@ -9384,10 +9390,10 @@
         <v>5</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="P65" s="2" t="s">
         <v>43</v>
@@ -9476,7 +9482,7 @@
     </row>
     <row r="66">
       <c r="A66" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>39</v>
@@ -9497,7 +9503,7 @@
         <v>10</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="P66" s="2" t="s">
         <v>43</v>
@@ -9586,7 +9592,7 @@
     </row>
     <row r="67">
       <c r="A67" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>39</v>
@@ -9607,7 +9613,7 @@
         <v>10</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P67" s="2" t="s">
         <v>43</v>
@@ -9830,13 +9836,13 @@
         <v>25</v>
       </c>
       <c r="AB1" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AC1" s="4" t="s">
         <v>29</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AE1" s="4" t="s">
         <v>31</v>
@@ -9845,12 +9851,12 @@
         <v>33</v>
       </c>
       <c r="AG1" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>39</v>
@@ -9871,13 +9877,13 @@
         <v>60</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>43</v>
@@ -9936,7 +9942,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>39</v>
@@ -9957,13 +9963,13 @@
         <v>60</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>43</v>
@@ -10022,7 +10028,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>39</v>
@@ -10043,16 +10049,16 @@
         <v>60</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>43</v>
@@ -10111,7 +10117,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>46</v>
@@ -10135,16 +10141,16 @@
         <v>8</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>81</v>
@@ -10206,7 +10212,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>39</v>
@@ -10227,13 +10233,13 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>81</v>
@@ -10295,7 +10301,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>62</v>
@@ -10319,13 +10325,13 @@
         <v>8</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>44</v>
@@ -10384,7 +10390,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>39</v>
@@ -10405,10 +10411,10 @@
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="P8" s="2" t="s">
         <v>43</v>
@@ -10467,7 +10473,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>39</v>
@@ -10488,13 +10494,13 @@
         <v>50</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>81</v>
@@ -10556,7 +10562,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>39</v>
@@ -10577,13 +10583,13 @@
         <v>50</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>81</v>
@@ -10645,7 +10651,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>39</v>
@@ -10666,16 +10672,16 @@
         <v>40</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>43</v>
@@ -10734,7 +10740,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>62</v>
@@ -10758,16 +10764,16 @@
         <v>9</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>43</v>
@@ -10826,7 +10832,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>39</v>
@@ -10847,13 +10853,13 @@
         <v>40</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>95</v>
@@ -10915,7 +10921,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>39</v>
@@ -10936,16 +10942,16 @@
         <v>30</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>43</v>
@@ -11004,7 +11010,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>39</v>
@@ -11025,19 +11031,19 @@
         <v>40</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="O15" s="3" t="s">
         <v>81</v>
@@ -11099,7 +11105,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>39</v>
@@ -11120,13 +11126,13 @@
         <v>45</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>81</v>
@@ -11188,7 +11194,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>39</v>
@@ -11209,13 +11215,13 @@
         <v>55</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>81</v>
@@ -11277,7 +11283,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>39</v>
@@ -11298,13 +11304,13 @@
         <v>20</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>43</v>
@@ -11363,7 +11369,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>39</v>
@@ -11384,13 +11390,13 @@
         <v>40</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>81</v>
@@ -11452,7 +11458,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>46</v>
@@ -11476,16 +11482,16 @@
         <v>6</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>43</v>
@@ -11544,7 +11550,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>39</v>
@@ -11565,13 +11571,13 @@
         <v>40</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>81</v>
@@ -11633,7 +11639,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>39</v>
@@ -11654,16 +11660,16 @@
         <v>45</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>43</v>
@@ -11722,7 +11728,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>39</v>
@@ -11743,16 +11749,16 @@
         <v>42</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>43</v>
@@ -11811,7 +11817,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>39</v>
@@ -11832,13 +11838,13 @@
         <v>50</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>81</v>
@@ -11900,7 +11906,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>39</v>
@@ -11921,16 +11927,16 @@
         <v>45</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>43</v>
@@ -11989,7 +11995,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>39</v>
@@ -12010,13 +12016,13 @@
         <v>45</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>43</v>
@@ -12075,7 +12081,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>39</v>
@@ -12096,16 +12102,16 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>95</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>43</v>
@@ -12164,7 +12170,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>39</v>
@@ -12185,19 +12191,19 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>43</v>
@@ -12256,7 +12262,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>39</v>
@@ -12277,16 +12283,16 @@
         <v>45</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>43</v>
@@ -12458,16 +12464,16 @@
         <v>21</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>23</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="Y1" s="4" t="s">
         <v>31</v>
@@ -12475,7 +12481,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>39</v>
@@ -12496,16 +12502,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>43</v>
@@ -12540,7 +12546,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>39</v>
@@ -12561,13 +12567,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>43</v>
@@ -12602,7 +12608,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>62</v>
@@ -12626,19 +12632,19 @@
         <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>43</v>
@@ -12673,7 +12679,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>39</v>
@@ -12694,16 +12700,16 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>43</v>
@@ -12738,7 +12744,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>39</v>
@@ -12759,16 +12765,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="L6" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="M6" s="3" t="s">
         <v>275</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>274</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>44</v>
@@ -12803,7 +12809,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>39</v>
@@ -12824,16 +12830,16 @@
         <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>44</v>
@@ -12868,7 +12874,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>46</v>
@@ -12892,16 +12898,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>44</v>
@@ -12936,7 +12942,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>39</v>
@@ -12957,19 +12963,19 @@
         <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>43</v>
@@ -13004,7 +13010,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>46</v>
@@ -13028,16 +13034,16 @@
         <v>10</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>43</v>
@@ -13072,7 +13078,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>62</v>
@@ -13096,13 +13102,13 @@
         <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>43</v>
@@ -13137,7 +13143,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>46</v>
@@ -13161,19 +13167,19 @@
         <v>9</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>43</v>
@@ -13208,7 +13214,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>39</v>
@@ -13229,19 +13235,19 @@
         <v>30</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P13" s="2" t="s">
         <v>43</v>
@@ -13276,7 +13282,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>39</v>
@@ -13297,19 +13303,19 @@
         <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>43</v>
@@ -13344,7 +13350,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>39</v>
@@ -13365,16 +13371,16 @@
         <v>30</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>44</v>
@@ -13409,7 +13415,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>39</v>
@@ -13430,19 +13436,19 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>43</v>
@@ -13477,7 +13483,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>39</v>
@@ -13498,16 +13504,16 @@
         <v>35</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>43</v>
@@ -13542,7 +13548,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>39</v>
@@ -13563,16 +13569,16 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P18" s="1" t="s">
         <v>44</v>
@@ -13607,7 +13613,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>39</v>
@@ -13628,16 +13634,16 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>44</v>
@@ -13672,7 +13678,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>39</v>
@@ -13693,16 +13699,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>44</v>
@@ -13737,7 +13743,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>39</v>
@@ -13758,16 +13764,16 @@
         <v>35</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>44</v>
@@ -13802,7 +13808,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>39</v>
@@ -13823,16 +13829,16 @@
         <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="P22" s="1" t="s">
         <v>44</v>
@@ -13867,7 +13873,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>46</v>
@@ -13891,16 +13897,16 @@
         <v>8</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>99</v>
@@ -13938,7 +13944,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>39</v>
@@ -13959,13 +13965,13 @@
         <v>20</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>43</v>
@@ -14000,7 +14006,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>39</v>
@@ -14021,16 +14027,16 @@
         <v>30</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>43</v>
@@ -14065,7 +14071,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>39</v>
@@ -14086,13 +14092,13 @@
         <v>35</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>44</v>
@@ -14127,7 +14133,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>39</v>
@@ -14148,16 +14154,16 @@
         <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>44</v>
@@ -14192,7 +14198,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>46</v>
@@ -14216,16 +14222,16 @@
         <v>16</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="P28" s="1" t="s">
         <v>44</v>
@@ -14361,16 +14367,16 @@
         <v>11</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>19</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>21</v>
@@ -14387,7 +14393,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>46</v>
@@ -14411,7 +14417,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>43</v>
@@ -14443,7 +14449,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>39</v>
@@ -14464,13 +14470,13 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>43</v>
@@ -14502,7 +14508,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>46</v>
@@ -14526,16 +14532,16 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>44</v>
@@ -14567,7 +14573,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>62</v>
@@ -14591,16 +14597,16 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>44</v>
@@ -14632,7 +14638,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>39</v>
@@ -14653,13 +14659,13 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>43</v>
@@ -14691,7 +14697,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>39</v>
@@ -14712,16 +14718,16 @@
         <v>35</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>44</v>
@@ -14753,7 +14759,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>39</v>
@@ -14774,16 +14780,16 @@
         <v>45</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>81</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>44</v>
@@ -14815,7 +14821,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>46</v>
@@ -14839,16 +14845,16 @@
         <v>8</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>44</v>
@@ -14880,7 +14886,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>39</v>
@@ -14901,16 +14907,16 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>43</v>
@@ -14942,7 +14948,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>39</v>
@@ -14963,19 +14969,19 @@
         <v>45</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>43</v>
@@ -15007,7 +15013,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>39</v>
@@ -15028,16 +15034,16 @@
         <v>37</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="P12" s="1" t="s">
         <v>44</v>
@@ -15069,7 +15075,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>39</v>
@@ -15096,10 +15102,10 @@
         <v>52</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="P13" s="2" t="s">
         <v>43</v>
@@ -15131,7 +15137,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>62</v>
@@ -15155,13 +15161,13 @@
         <v>12</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>43</v>
@@ -15193,7 +15199,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>46</v>
@@ -15217,16 +15223,16 @@
         <v>9</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>43</v>
@@ -15258,7 +15264,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>39</v>
@@ -15279,19 +15285,19 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>95</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="P16" s="1" t="s">
         <v>44</v>
@@ -15323,7 +15329,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>39</v>
@@ -15344,16 +15350,16 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>43</v>
@@ -15385,7 +15391,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>39</v>
@@ -15406,19 +15412,19 @@
         <v>41</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>43</v>
@@ -15450,7 +15456,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>39</v>
@@ -15471,19 +15477,19 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>44</v>
@@ -15515,7 +15521,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>39</v>
@@ -15536,16 +15542,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>44</v>
@@ -15577,7 +15583,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>39</v>
@@ -15598,13 +15604,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>43</v>
@@ -15636,7 +15642,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>39</v>
@@ -15657,16 +15663,16 @@
         <v>31</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>43</v>
@@ -15698,7 +15704,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>39</v>
@@ -15719,13 +15725,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>43</v>
@@ -15757,7 +15763,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>39</v>
@@ -15778,7 +15784,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>44</v>
@@ -15810,7 +15816,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>39</v>
@@ -15831,16 +15837,16 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="P25" s="1" t="s">
         <v>44</v>
@@ -15872,7 +15878,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>39</v>
@@ -15893,13 +15899,13 @@
         <v>24</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>43</v>
@@ -15931,7 +15937,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>39</v>
@@ -15952,13 +15958,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>44</v>
@@ -15990,7 +15996,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>39</v>
@@ -16011,13 +16017,13 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>43</v>
@@ -16049,7 +16055,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>39</v>
@@ -16070,16 +16076,16 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>43</v>
@@ -16111,7 +16117,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>46</v>
@@ -16135,16 +16141,16 @@
         <v>8</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>43</v>
@@ -16176,7 +16182,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>39</v>
@@ -16197,13 +16203,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>43</v>
@@ -16235,7 +16241,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>39</v>
@@ -16256,13 +16262,13 @@
         <v>45</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>43</v>
@@ -16294,7 +16300,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>39</v>
@@ -16315,13 +16321,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>44</v>
@@ -16353,7 +16359,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>39</v>
@@ -16374,13 +16380,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>44</v>
@@ -16412,7 +16418,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>39</v>
@@ -16433,13 +16439,13 @@
         <v>45</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>43</v>
@@ -16471,7 +16477,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>46</v>
@@ -16495,16 +16501,16 @@
         <v>7</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="P36" s="1" t="s">
         <v>44</v>
@@ -16643,24 +16649,24 @@
         <v>18</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>31</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>46</v>
@@ -16684,16 +16690,16 @@
         <v>6</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>44</v>
@@ -16722,7 +16728,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>39</v>
@@ -16743,13 +16749,13 @@
         <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>44</v>

</xml_diff>